<commit_message>
Update 3 Auswertung Photometrie.xlsx
</commit_message>
<xml_diff>
--- a/Wasser/3 Auswertung Photometrie.xlsx
+++ b/Wasser/3 Auswertung Photometrie.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alexandra\Documents\GitHub\Moore-Lichtenau-Meusebach\Wasser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3231E15E-B60A-4156-9407-8CFB913B5C98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D0C6AF8-268B-413D-8063-FBADAB4F566B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="26.06.2025" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="31.08.2025" sheetId="3" r:id="rId3"/>
     <sheet name="24.09.2025" sheetId="5" r:id="rId4"/>
     <sheet name="Zusammenfassung" sheetId="7" r:id="rId5"/>
+    <sheet name="Ergebnisse" sheetId="8" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="126">
   <si>
     <t>sample</t>
   </si>
@@ -383,13 +384,50 @@
   <si>
     <t>Ammonium</t>
   </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>L2</t>
+  </si>
+  <si>
+    <t>L3</t>
+  </si>
+  <si>
+    <t>L4</t>
+  </si>
+  <si>
+    <t>MN1</t>
+  </si>
+  <si>
+    <t>MN2</t>
+  </si>
+  <si>
+    <t>MN3</t>
+  </si>
+  <si>
+    <t>MT1</t>
+  </si>
+  <si>
+    <t>MT2</t>
+  </si>
+  <si>
+    <t>Messstelle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mittelwerte je Fläche </t>
+  </si>
+  <si>
+    <t>Mittelwerte je Logger</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="168" formatCode="0.0000"/>
   </numFmts>
   <fonts count="20" x14ac:knownFonts="1">
     <font>
@@ -1479,7 +1517,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1546,16 +1584,43 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1570,54 +1635,6 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1630,13 +1647,40 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1645,12 +1689,8 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="2" fontId="0" fillId="33" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20 % - Akzent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -14655,16 +14695,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
       <c r="I1" s="1"/>
     </row>
     <row r="2" spans="1:9" s="25" customFormat="1" x14ac:dyDescent="0.25">
@@ -14870,14 +14910,14 @@
       <c r="B55" s="4">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="C55" s="77">
+      <c r="C55" s="52">
         <v>1</v>
       </c>
-      <c r="D55" s="77"/>
-      <c r="E55" s="68">
+      <c r="D55" s="52"/>
+      <c r="E55" s="53">
         <v>0</v>
       </c>
-      <c r="F55" s="69"/>
+      <c r="F55" s="54"/>
       <c r="H55" s="18"/>
       <c r="I55" s="27"/>
       <c r="J55" s="18"/>
@@ -14889,15 +14929,15 @@
       <c r="B56" s="6">
         <v>1.6E-2</v>
       </c>
-      <c r="C56" s="76">
+      <c r="C56" s="49">
         <v>2.5</v>
       </c>
-      <c r="D56" s="76"/>
-      <c r="E56" s="57">
+      <c r="D56" s="49"/>
+      <c r="E56" s="55">
         <f t="shared" ref="E56" si="0">(B56-0.0164)/0.0093</f>
         <v>-4.3010752688172157E-2</v>
       </c>
-      <c r="F56" s="58"/>
+      <c r="F56" s="56"/>
       <c r="H56" s="18"/>
       <c r="I56" s="27"/>
       <c r="J56" s="18"/>
@@ -14909,15 +14949,15 @@
       <c r="B57" s="6">
         <v>0.04</v>
       </c>
-      <c r="C57" s="76">
+      <c r="C57" s="49">
         <v>5</v>
       </c>
-      <c r="D57" s="76"/>
-      <c r="E57" s="57">
+      <c r="D57" s="49"/>
+      <c r="E57" s="55">
         <f>(B57-0.0164)/0.0093</f>
         <v>2.5376344086021505</v>
       </c>
-      <c r="F57" s="58"/>
+      <c r="F57" s="56"/>
       <c r="H57" s="18">
         <f>C57/1000000</f>
         <v>5.0000000000000004E-6</v>
@@ -14938,10 +14978,10 @@
       <c r="B58" s="6">
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="C58" s="76">
+      <c r="C58" s="49">
         <v>10</v>
       </c>
-      <c r="D58" s="76"/>
+      <c r="D58" s="49"/>
       <c r="E58" s="50">
         <f t="shared" ref="E58:E62" si="1">(B58-0.0164)/0.0093</f>
         <v>7.2688172043010768</v>
@@ -14967,10 +15007,10 @@
       <c r="B59" s="6">
         <v>0.22800000000000001</v>
       </c>
-      <c r="C59" s="76">
+      <c r="C59" s="49">
         <v>25</v>
       </c>
-      <c r="D59" s="76"/>
+      <c r="D59" s="49"/>
       <c r="E59" s="50">
         <f t="shared" si="1"/>
         <v>22.752688172043015</v>
@@ -14987,10 +15027,10 @@
       <c r="B60" s="6">
         <v>0.54300000000000004</v>
       </c>
-      <c r="C60" s="76">
+      <c r="C60" s="49">
         <v>50</v>
       </c>
-      <c r="D60" s="76"/>
+      <c r="D60" s="49"/>
       <c r="E60" s="50">
         <f t="shared" si="1"/>
         <v>56.62365591397851</v>
@@ -15016,10 +15056,10 @@
       <c r="B61" s="6">
         <v>0.98199999999999998</v>
       </c>
-      <c r="C61" s="76">
+      <c r="C61" s="49">
         <v>100</v>
       </c>
-      <c r="D61" s="76"/>
+      <c r="D61" s="49"/>
       <c r="E61" s="50">
         <f t="shared" si="1"/>
         <v>103.82795698924733</v>
@@ -15045,15 +15085,15 @@
       <c r="B62" s="8">
         <v>1.8460000000000001</v>
       </c>
-      <c r="C62" s="52">
+      <c r="C62" s="61">
         <v>200</v>
       </c>
-      <c r="D62" s="53"/>
-      <c r="E62" s="54">
+      <c r="D62" s="62"/>
+      <c r="E62" s="63">
         <f t="shared" si="1"/>
         <v>196.73118279569894</v>
       </c>
-      <c r="F62" s="55"/>
+      <c r="F62" s="64"/>
       <c r="H62" s="19">
         <f>C62/1000000</f>
         <v>2.0000000000000001E-4</v>
@@ -15074,12 +15114,12 @@
       <c r="B63" s="9">
         <v>1.0999999999999999E-2</v>
       </c>
-      <c r="C63" s="72"/>
-      <c r="D63" s="73"/>
-      <c r="E63" s="74">
+      <c r="C63" s="65"/>
+      <c r="D63" s="66"/>
+      <c r="E63" s="67">
         <v>0</v>
       </c>
-      <c r="F63" s="75"/>
+      <c r="F63" s="68"/>
       <c r="H63" s="18">
         <f t="shared" ref="H63:H70" si="4">E63/1000000</f>
         <v>0</v>
@@ -15100,12 +15140,12 @@
       <c r="B64" s="6">
         <v>2E-3</v>
       </c>
-      <c r="C64" s="48"/>
-      <c r="D64" s="56"/>
-      <c r="E64" s="57">
+      <c r="C64" s="59"/>
+      <c r="D64" s="60"/>
+      <c r="E64" s="55">
         <v>0</v>
       </c>
-      <c r="F64" s="58"/>
+      <c r="F64" s="56"/>
       <c r="H64" s="18">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -15126,12 +15166,12 @@
       <c r="B65" s="6">
         <v>2E-3</v>
       </c>
-      <c r="C65" s="48"/>
-      <c r="D65" s="56"/>
-      <c r="E65" s="57">
+      <c r="C65" s="59"/>
+      <c r="D65" s="60"/>
+      <c r="E65" s="55">
         <v>0</v>
       </c>
-      <c r="F65" s="58"/>
+      <c r="F65" s="56"/>
       <c r="H65" s="18">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -15152,12 +15192,12 @@
       <c r="B66" s="6">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="C66" s="48"/>
-      <c r="D66" s="56"/>
-      <c r="E66" s="57">
+      <c r="C66" s="59"/>
+      <c r="D66" s="60"/>
+      <c r="E66" s="55">
         <v>0</v>
       </c>
-      <c r="F66" s="58"/>
+      <c r="F66" s="56"/>
       <c r="H66" s="18">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -15178,13 +15218,13 @@
       <c r="B67" s="6">
         <v>0.109</v>
       </c>
-      <c r="C67" s="48"/>
-      <c r="D67" s="56"/>
-      <c r="E67" s="57">
+      <c r="C67" s="59"/>
+      <c r="D67" s="60"/>
+      <c r="E67" s="55">
         <f t="shared" ref="E67:E70" si="7">(B67-0.0164)/0.0093</f>
         <v>9.9569892473118298</v>
       </c>
-      <c r="F67" s="58"/>
+      <c r="F67" s="56"/>
       <c r="H67" s="18">
         <f t="shared" si="4"/>
         <v>9.9569892473118294E-6</v>
@@ -15205,13 +15245,13 @@
       <c r="B68" s="6">
         <v>0.36</v>
       </c>
-      <c r="C68" s="48"/>
-      <c r="D68" s="56"/>
-      <c r="E68" s="57">
+      <c r="C68" s="59"/>
+      <c r="D68" s="60"/>
+      <c r="E68" s="55">
         <f t="shared" si="7"/>
         <v>36.946236559139784</v>
       </c>
-      <c r="F68" s="58"/>
+      <c r="F68" s="56"/>
       <c r="H68" s="18">
         <f t="shared" si="4"/>
         <v>3.6946236559139785E-5</v>
@@ -15232,13 +15272,13 @@
       <c r="B69" s="6">
         <v>0.91300000000000003</v>
       </c>
-      <c r="C69" s="48"/>
-      <c r="D69" s="56"/>
-      <c r="E69" s="57">
+      <c r="C69" s="59"/>
+      <c r="D69" s="60"/>
+      <c r="E69" s="55">
         <f t="shared" si="7"/>
         <v>96.408602150537646</v>
       </c>
-      <c r="F69" s="58"/>
+      <c r="F69" s="56"/>
       <c r="H69" s="18">
         <f t="shared" si="4"/>
         <v>9.6408602150537646E-5</v>
@@ -15259,13 +15299,13 @@
       <c r="B70" s="8">
         <v>4.7E-2</v>
       </c>
-      <c r="C70" s="52"/>
-      <c r="D70" s="59"/>
-      <c r="E70" s="60">
+      <c r="C70" s="61"/>
+      <c r="D70" s="69"/>
+      <c r="E70" s="57">
         <f t="shared" si="7"/>
         <v>3.2903225806451615</v>
       </c>
-      <c r="F70" s="61"/>
+      <c r="F70" s="58"/>
       <c r="H70" s="18">
         <f t="shared" si="4"/>
         <v>3.2903225806451615E-6</v>
@@ -15350,11 +15390,11 @@
         <v>0.5</v>
       </c>
       <c r="D101" s="11"/>
-      <c r="E101" s="68">
+      <c r="E101" s="53">
         <f>(B101+0.0049)/0.0204</f>
         <v>0.28921568627450978</v>
       </c>
-      <c r="F101" s="69"/>
+      <c r="F101" s="54"/>
       <c r="I101" s="16">
         <f t="shared" ref="I101:I106" si="8">C101/1000000</f>
         <v>4.9999999999999998E-7</v>
@@ -15379,11 +15419,11 @@
         <v>1</v>
       </c>
       <c r="D102" s="13"/>
-      <c r="E102" s="57">
+      <c r="E102" s="55">
         <f t="shared" ref="E102:E106" si="10">(B102+0.0049)/0.0204</f>
         <v>1.0245098039215685</v>
       </c>
-      <c r="F102" s="58"/>
+      <c r="F102" s="56"/>
       <c r="I102" s="18">
         <f t="shared" si="8"/>
         <v>9.9999999999999995E-7</v>
@@ -15408,11 +15448,11 @@
         <v>5</v>
       </c>
       <c r="D103" s="13"/>
-      <c r="E103" s="57">
+      <c r="E103" s="55">
         <f t="shared" si="10"/>
         <v>4.6029411764705879</v>
       </c>
-      <c r="F103" s="58"/>
+      <c r="F103" s="56"/>
       <c r="I103" s="18">
         <f t="shared" si="8"/>
         <v>5.0000000000000004E-6</v>
@@ -15437,11 +15477,11 @@
         <v>10</v>
       </c>
       <c r="D104" s="13"/>
-      <c r="E104" s="57">
+      <c r="E104" s="55">
         <f t="shared" si="10"/>
         <v>10.877450980392155</v>
       </c>
-      <c r="F104" s="58"/>
+      <c r="F104" s="56"/>
       <c r="I104" s="18">
         <f t="shared" si="8"/>
         <v>1.0000000000000001E-5</v>
@@ -15466,11 +15506,11 @@
         <v>25</v>
       </c>
       <c r="D105" s="33"/>
-      <c r="E105" s="57">
+      <c r="E105" s="55">
         <f t="shared" si="10"/>
         <v>24.799019607843135</v>
       </c>
-      <c r="F105" s="58"/>
+      <c r="F105" s="56"/>
       <c r="I105" s="18">
         <f t="shared" si="8"/>
         <v>2.5000000000000001E-5</v>
@@ -15495,11 +15535,11 @@
         <v>50</v>
       </c>
       <c r="D106" s="15"/>
-      <c r="E106" s="60">
+      <c r="E106" s="57">
         <f t="shared" si="10"/>
         <v>37.446078431372548</v>
       </c>
-      <c r="F106" s="61"/>
+      <c r="F106" s="58"/>
       <c r="I106" s="19">
         <f t="shared" si="8"/>
         <v>5.0000000000000002E-5</v>
@@ -15520,13 +15560,13 @@
       <c r="B107" s="4">
         <v>0</v>
       </c>
-      <c r="C107" s="62"/>
+      <c r="C107" s="70"/>
       <c r="D107" s="71"/>
-      <c r="E107" s="68">
+      <c r="E107" s="53">
         <f t="shared" ref="E107" si="12">(B107+0.0049)/0.0204</f>
         <v>0.24019607843137253</v>
       </c>
-      <c r="F107" s="69"/>
+      <c r="F107" s="54"/>
       <c r="I107" s="18">
         <f>E107/1000000</f>
         <v>2.4019607843137255E-7</v>
@@ -15547,13 +15587,13 @@
       <c r="B108" s="6">
         <v>0</v>
       </c>
-      <c r="C108" s="48"/>
-      <c r="D108" s="56"/>
-      <c r="E108" s="57">
+      <c r="C108" s="59"/>
+      <c r="D108" s="60"/>
+      <c r="E108" s="55">
         <f t="shared" ref="E108:E114" si="13">(B108+0.0049)/0.0204</f>
         <v>0.24019607843137253</v>
       </c>
-      <c r="F108" s="58"/>
+      <c r="F108" s="56"/>
       <c r="I108" s="18">
         <f t="shared" ref="I108:I114" si="14">E108/1000000</f>
         <v>2.4019607843137255E-7</v>
@@ -15574,13 +15614,13 @@
       <c r="B109" s="6">
         <v>0</v>
       </c>
-      <c r="C109" s="48"/>
-      <c r="D109" s="56"/>
-      <c r="E109" s="57">
+      <c r="C109" s="59"/>
+      <c r="D109" s="60"/>
+      <c r="E109" s="55">
         <f t="shared" si="13"/>
         <v>0.24019607843137253</v>
       </c>
-      <c r="F109" s="58"/>
+      <c r="F109" s="56"/>
       <c r="I109" s="18">
         <f t="shared" si="14"/>
         <v>2.4019607843137255E-7</v>
@@ -15601,13 +15641,13 @@
       <c r="B110" s="6">
         <v>0</v>
       </c>
-      <c r="C110" s="48"/>
-      <c r="D110" s="56"/>
-      <c r="E110" s="57">
+      <c r="C110" s="59"/>
+      <c r="D110" s="60"/>
+      <c r="E110" s="55">
         <f t="shared" si="13"/>
         <v>0.24019607843137253</v>
       </c>
-      <c r="F110" s="58"/>
+      <c r="F110" s="56"/>
       <c r="I110" s="18">
         <f t="shared" si="14"/>
         <v>2.4019607843137255E-7</v>
@@ -15628,13 +15668,13 @@
       <c r="B111" s="6">
         <v>1.4E-2</v>
       </c>
-      <c r="C111" s="48"/>
-      <c r="D111" s="56"/>
-      <c r="E111" s="57">
+      <c r="C111" s="59"/>
+      <c r="D111" s="60"/>
+      <c r="E111" s="55">
         <f t="shared" si="13"/>
         <v>0.92647058823529405</v>
       </c>
-      <c r="F111" s="58"/>
+      <c r="F111" s="56"/>
       <c r="I111" s="18">
         <f t="shared" si="14"/>
         <v>9.2647058823529408E-7</v>
@@ -15655,13 +15695,13 @@
       <c r="B112" s="6">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="C112" s="48"/>
-      <c r="D112" s="56"/>
-      <c r="E112" s="57">
+      <c r="C112" s="59"/>
+      <c r="D112" s="60"/>
+      <c r="E112" s="55">
         <f t="shared" si="13"/>
         <v>0.68137254901960775</v>
       </c>
-      <c r="F112" s="58"/>
+      <c r="F112" s="56"/>
       <c r="I112" s="18">
         <f t="shared" si="14"/>
         <v>6.8137254901960776E-7</v>
@@ -15682,13 +15722,13 @@
       <c r="B113" s="6">
         <v>3.9E-2</v>
       </c>
-      <c r="C113" s="48"/>
-      <c r="D113" s="56"/>
-      <c r="E113" s="57">
+      <c r="C113" s="59"/>
+      <c r="D113" s="60"/>
+      <c r="E113" s="55">
         <f t="shared" si="13"/>
         <v>2.1519607843137254</v>
       </c>
-      <c r="F113" s="58"/>
+      <c r="F113" s="56"/>
       <c r="I113" s="18">
         <f t="shared" si="14"/>
         <v>2.1519607843137253E-6</v>
@@ -15709,13 +15749,13 @@
       <c r="B114" s="8">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="C114" s="52"/>
-      <c r="D114" s="59"/>
-      <c r="E114" s="60">
+      <c r="C114" s="61"/>
+      <c r="D114" s="69"/>
+      <c r="E114" s="57">
         <f t="shared" si="13"/>
         <v>0.53431372549019607</v>
       </c>
-      <c r="F114" s="61"/>
+      <c r="F114" s="58"/>
       <c r="I114" s="18">
         <f t="shared" si="14"/>
         <v>5.3431372549019611E-7</v>
@@ -15747,16 +15787,16 @@
       </c>
     </row>
     <row r="120" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A120" s="70" t="s">
+      <c r="A120" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="B120" s="70"/>
-      <c r="C120" s="70"/>
-      <c r="D120" s="70"/>
-      <c r="E120" s="70"/>
-      <c r="F120" s="70"/>
-      <c r="G120" s="70"/>
-      <c r="H120" s="70"/>
+      <c r="B120" s="48"/>
+      <c r="C120" s="48"/>
+      <c r="D120" s="48"/>
+      <c r="E120" s="48"/>
+      <c r="F120" s="48"/>
+      <c r="G120" s="48"/>
+      <c r="H120" s="48"/>
     </row>
     <row r="121" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I121" s="16" t="s">
@@ -15802,14 +15842,14 @@
       <c r="B123" s="4">
         <v>0</v>
       </c>
-      <c r="C123" s="62">
+      <c r="C123" s="70">
         <v>2.5</v>
       </c>
-      <c r="D123" s="63"/>
-      <c r="E123" s="68">
+      <c r="D123" s="72"/>
+      <c r="E123" s="53">
         <v>0</v>
       </c>
-      <c r="F123" s="69"/>
+      <c r="F123" s="54"/>
       <c r="G123" s="35"/>
       <c r="I123" s="16">
         <f t="shared" ref="I123:I130" si="17">C123/1000000</f>
@@ -15831,10 +15871,10 @@
       <c r="B124" s="2">
         <v>1E-3</v>
       </c>
-      <c r="C124" s="66">
+      <c r="C124" s="76">
         <v>5</v>
       </c>
-      <c r="D124" s="67"/>
+      <c r="D124" s="77"/>
       <c r="E124" s="50">
         <f t="shared" ref="E124:E130" si="18">(B124+0.0067)/0.0019</f>
         <v>4.0526315789473681</v>
@@ -15861,10 +15901,10 @@
       <c r="B125" s="6">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="C125" s="48">
+      <c r="C125" s="59">
         <v>10</v>
       </c>
-      <c r="D125" s="49"/>
+      <c r="D125" s="75"/>
       <c r="E125" s="50">
         <f t="shared" si="18"/>
         <v>7.7368421052631584</v>
@@ -15891,10 +15931,10 @@
       <c r="B126" s="6">
         <v>4.1000000000000002E-2</v>
       </c>
-      <c r="C126" s="48">
+      <c r="C126" s="59">
         <v>25</v>
       </c>
-      <c r="D126" s="49"/>
+      <c r="D126" s="75"/>
       <c r="E126" s="50">
         <f t="shared" si="18"/>
         <v>25.105263157894736</v>
@@ -15921,10 +15961,10 @@
       <c r="B127" s="6">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="C127" s="48">
+      <c r="C127" s="59">
         <v>50</v>
       </c>
-      <c r="D127" s="49"/>
+      <c r="D127" s="75"/>
       <c r="E127" s="50">
         <f t="shared" si="18"/>
         <v>47.210526315789473</v>
@@ -15951,10 +15991,10 @@
       <c r="B128" s="6">
         <v>0.17499999999999999</v>
       </c>
-      <c r="C128" s="48">
+      <c r="C128" s="59">
         <v>100</v>
       </c>
-      <c r="D128" s="49"/>
+      <c r="D128" s="75"/>
       <c r="E128" s="50">
         <f t="shared" si="18"/>
         <v>95.631578947368425</v>
@@ -15981,10 +16021,10 @@
       <c r="B129" s="6">
         <v>0.375</v>
       </c>
-      <c r="C129" s="48">
+      <c r="C129" s="59">
         <v>200</v>
       </c>
-      <c r="D129" s="49"/>
+      <c r="D129" s="75"/>
       <c r="E129" s="50">
         <f t="shared" si="18"/>
         <v>200.89473684210526</v>
@@ -16011,15 +16051,15 @@
       <c r="B130" s="8">
         <v>0.91500000000000004</v>
       </c>
-      <c r="C130" s="52">
+      <c r="C130" s="61">
         <v>500</v>
       </c>
-      <c r="D130" s="53"/>
-      <c r="E130" s="54">
+      <c r="D130" s="62"/>
+      <c r="E130" s="63">
         <f t="shared" si="18"/>
         <v>485.1052631578948</v>
       </c>
-      <c r="F130" s="55"/>
+      <c r="F130" s="64"/>
       <c r="G130" s="35"/>
       <c r="I130" s="19">
         <f t="shared" si="17"/>
@@ -16041,13 +16081,13 @@
       <c r="B131" s="4">
         <v>1.0999999999999999E-2</v>
       </c>
-      <c r="C131" s="62"/>
-      <c r="D131" s="63"/>
-      <c r="E131" s="64">
+      <c r="C131" s="70"/>
+      <c r="D131" s="72"/>
+      <c r="E131" s="73">
         <f t="shared" ref="E131:E138" si="21">(B131+0.0067)/0.0019</f>
         <v>9.3157894736842106</v>
       </c>
-      <c r="F131" s="65"/>
+      <c r="F131" s="74"/>
       <c r="G131" s="35"/>
       <c r="I131" s="18">
         <f>E131/1000000</f>
@@ -16069,8 +16109,8 @@
       <c r="B132" s="6">
         <v>0</v>
       </c>
-      <c r="C132" s="48"/>
-      <c r="D132" s="49"/>
+      <c r="C132" s="59"/>
+      <c r="D132" s="75"/>
       <c r="E132" s="50">
         <v>0</v>
       </c>
@@ -16096,8 +16136,8 @@
       <c r="B133" s="6">
         <v>0</v>
       </c>
-      <c r="C133" s="48"/>
-      <c r="D133" s="49"/>
+      <c r="C133" s="59"/>
+      <c r="D133" s="75"/>
       <c r="E133" s="50">
         <v>0</v>
       </c>
@@ -16123,8 +16163,8 @@
       <c r="B134" s="6">
         <v>0</v>
       </c>
-      <c r="C134" s="48"/>
-      <c r="D134" s="49"/>
+      <c r="C134" s="59"/>
+      <c r="D134" s="75"/>
       <c r="E134" s="50">
         <v>0</v>
       </c>
@@ -16150,8 +16190,8 @@
       <c r="B135" s="6">
         <v>0</v>
       </c>
-      <c r="C135" s="48"/>
-      <c r="D135" s="49"/>
+      <c r="C135" s="59"/>
+      <c r="D135" s="75"/>
       <c r="E135" s="50">
         <v>0</v>
       </c>
@@ -16177,8 +16217,8 @@
       <c r="B136" s="6">
         <v>1.7999999999999999E-2</v>
       </c>
-      <c r="C136" s="48"/>
-      <c r="D136" s="49"/>
+      <c r="C136" s="59"/>
+      <c r="D136" s="75"/>
       <c r="E136" s="50">
         <f t="shared" si="21"/>
         <v>13</v>
@@ -16205,8 +16245,8 @@
       <c r="B137" s="6">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="C137" s="48"/>
-      <c r="D137" s="49"/>
+      <c r="C137" s="59"/>
+      <c r="D137" s="75"/>
       <c r="E137" s="50">
         <f t="shared" si="21"/>
         <v>18.263157894736842</v>
@@ -16233,13 +16273,13 @@
       <c r="B138" s="8">
         <v>2.7E-2</v>
       </c>
-      <c r="C138" s="52"/>
-      <c r="D138" s="53"/>
-      <c r="E138" s="54">
+      <c r="C138" s="61"/>
+      <c r="D138" s="62"/>
+      <c r="E138" s="63">
         <f t="shared" si="21"/>
         <v>17.736842105263158</v>
       </c>
-      <c r="F138" s="55"/>
+      <c r="F138" s="64"/>
       <c r="G138" s="35"/>
       <c r="I138" s="18">
         <f t="shared" si="24"/>
@@ -16256,13 +16296,71 @@
     </row>
   </sheetData>
   <mergeCells count="88">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="C59:D59"/>
-    <mergeCell ref="E59:F59"/>
-    <mergeCell ref="C56:D56"/>
-    <mergeCell ref="C55:D55"/>
-    <mergeCell ref="E55:F55"/>
-    <mergeCell ref="E56:F56"/>
+    <mergeCell ref="C137:D137"/>
+    <mergeCell ref="E137:F137"/>
+    <mergeCell ref="C138:D138"/>
+    <mergeCell ref="E138:F138"/>
+    <mergeCell ref="C132:D132"/>
+    <mergeCell ref="E132:F132"/>
+    <mergeCell ref="C133:D133"/>
+    <mergeCell ref="E133:F133"/>
+    <mergeCell ref="C134:D134"/>
+    <mergeCell ref="E134:F134"/>
+    <mergeCell ref="C135:D135"/>
+    <mergeCell ref="E135:F135"/>
+    <mergeCell ref="C136:D136"/>
+    <mergeCell ref="E136:F136"/>
+    <mergeCell ref="C128:D128"/>
+    <mergeCell ref="E128:F128"/>
+    <mergeCell ref="C129:D129"/>
+    <mergeCell ref="E129:F129"/>
+    <mergeCell ref="C130:D130"/>
+    <mergeCell ref="E130:F130"/>
+    <mergeCell ref="C113:D113"/>
+    <mergeCell ref="E113:F113"/>
+    <mergeCell ref="C114:D114"/>
+    <mergeCell ref="E114:F114"/>
+    <mergeCell ref="C131:D131"/>
+    <mergeCell ref="E131:F131"/>
+    <mergeCell ref="C126:D126"/>
+    <mergeCell ref="E126:F126"/>
+    <mergeCell ref="C124:D124"/>
+    <mergeCell ref="E124:F124"/>
+    <mergeCell ref="C123:D123"/>
+    <mergeCell ref="E123:F123"/>
+    <mergeCell ref="A120:H120"/>
+    <mergeCell ref="C125:D125"/>
+    <mergeCell ref="E125:F125"/>
+    <mergeCell ref="C127:D127"/>
+    <mergeCell ref="E127:F127"/>
+    <mergeCell ref="E101:F101"/>
+    <mergeCell ref="E102:F102"/>
+    <mergeCell ref="C69:D69"/>
+    <mergeCell ref="E69:F69"/>
+    <mergeCell ref="C70:D70"/>
+    <mergeCell ref="E70:F70"/>
+    <mergeCell ref="C112:D112"/>
+    <mergeCell ref="E112:F112"/>
+    <mergeCell ref="E103:F103"/>
+    <mergeCell ref="E104:F104"/>
+    <mergeCell ref="E105:F105"/>
+    <mergeCell ref="C107:D107"/>
+    <mergeCell ref="E107:F107"/>
+    <mergeCell ref="C108:D108"/>
+    <mergeCell ref="E108:F108"/>
+    <mergeCell ref="C109:D109"/>
+    <mergeCell ref="E109:F109"/>
+    <mergeCell ref="C110:D110"/>
+    <mergeCell ref="E110:F110"/>
+    <mergeCell ref="C111:D111"/>
+    <mergeCell ref="E111:F111"/>
+    <mergeCell ref="E68:F68"/>
+    <mergeCell ref="C63:D63"/>
+    <mergeCell ref="E63:F63"/>
+    <mergeCell ref="C64:D64"/>
+    <mergeCell ref="E64:F64"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="E65:F65"/>
     <mergeCell ref="E106:F106"/>
     <mergeCell ref="C57:D57"/>
     <mergeCell ref="E57:F57"/>
@@ -16279,71 +16377,13 @@
     <mergeCell ref="C67:D67"/>
     <mergeCell ref="E67:F67"/>
     <mergeCell ref="C68:D68"/>
-    <mergeCell ref="E68:F68"/>
-    <mergeCell ref="C63:D63"/>
-    <mergeCell ref="E63:F63"/>
-    <mergeCell ref="C64:D64"/>
-    <mergeCell ref="E64:F64"/>
-    <mergeCell ref="C65:D65"/>
-    <mergeCell ref="E65:F65"/>
-    <mergeCell ref="C109:D109"/>
-    <mergeCell ref="E109:F109"/>
-    <mergeCell ref="C110:D110"/>
-    <mergeCell ref="E110:F110"/>
-    <mergeCell ref="C111:D111"/>
-    <mergeCell ref="E111:F111"/>
-    <mergeCell ref="E127:F127"/>
-    <mergeCell ref="E101:F101"/>
-    <mergeCell ref="E102:F102"/>
-    <mergeCell ref="C69:D69"/>
-    <mergeCell ref="E69:F69"/>
-    <mergeCell ref="C70:D70"/>
-    <mergeCell ref="E70:F70"/>
-    <mergeCell ref="C112:D112"/>
-    <mergeCell ref="E112:F112"/>
-    <mergeCell ref="E103:F103"/>
-    <mergeCell ref="E104:F104"/>
-    <mergeCell ref="E105:F105"/>
-    <mergeCell ref="C107:D107"/>
-    <mergeCell ref="E107:F107"/>
-    <mergeCell ref="C108:D108"/>
-    <mergeCell ref="E108:F108"/>
-    <mergeCell ref="C113:D113"/>
-    <mergeCell ref="E113:F113"/>
-    <mergeCell ref="C114:D114"/>
-    <mergeCell ref="E114:F114"/>
-    <mergeCell ref="C131:D131"/>
-    <mergeCell ref="E131:F131"/>
-    <mergeCell ref="C126:D126"/>
-    <mergeCell ref="E126:F126"/>
-    <mergeCell ref="C124:D124"/>
-    <mergeCell ref="E124:F124"/>
-    <mergeCell ref="C123:D123"/>
-    <mergeCell ref="E123:F123"/>
-    <mergeCell ref="A120:H120"/>
-    <mergeCell ref="C125:D125"/>
-    <mergeCell ref="E125:F125"/>
-    <mergeCell ref="C127:D127"/>
-    <mergeCell ref="C128:D128"/>
-    <mergeCell ref="E128:F128"/>
-    <mergeCell ref="C129:D129"/>
-    <mergeCell ref="E129:F129"/>
-    <mergeCell ref="C130:D130"/>
-    <mergeCell ref="E130:F130"/>
-    <mergeCell ref="C137:D137"/>
-    <mergeCell ref="E137:F137"/>
-    <mergeCell ref="C138:D138"/>
-    <mergeCell ref="E138:F138"/>
-    <mergeCell ref="C132:D132"/>
-    <mergeCell ref="E132:F132"/>
-    <mergeCell ref="C133:D133"/>
-    <mergeCell ref="E133:F133"/>
-    <mergeCell ref="C134:D134"/>
-    <mergeCell ref="E134:F134"/>
-    <mergeCell ref="C135:D135"/>
-    <mergeCell ref="E135:F135"/>
-    <mergeCell ref="C136:D136"/>
-    <mergeCell ref="E136:F136"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="C59:D59"/>
+    <mergeCell ref="E59:F59"/>
+    <mergeCell ref="C56:D56"/>
+    <mergeCell ref="C55:D55"/>
+    <mergeCell ref="E55:F55"/>
+    <mergeCell ref="E56:F56"/>
   </mergeCells>
   <pageMargins left="0.11458333333333333" right="1.0416666666666666E-2" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -16366,16 +16406,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
       <c r="I1" s="1"/>
     </row>
     <row r="2" spans="1:9" s="25" customFormat="1" x14ac:dyDescent="0.25">
@@ -16579,14 +16619,14 @@
         <v>34</v>
       </c>
       <c r="B55" s="4"/>
-      <c r="C55" s="77">
+      <c r="C55" s="52">
         <v>1</v>
       </c>
-      <c r="D55" s="77"/>
-      <c r="E55" s="68">
+      <c r="D55" s="52"/>
+      <c r="E55" s="53">
         <v>0</v>
       </c>
-      <c r="F55" s="69"/>
+      <c r="F55" s="54"/>
       <c r="H55" s="18"/>
       <c r="I55" s="27"/>
       <c r="J55" s="18"/>
@@ -16596,15 +16636,15 @@
         <v>35</v>
       </c>
       <c r="B56" s="6"/>
-      <c r="C56" s="76">
+      <c r="C56" s="49">
         <v>2.5</v>
       </c>
-      <c r="D56" s="76"/>
-      <c r="E56" s="57">
+      <c r="D56" s="49"/>
+      <c r="E56" s="55">
         <f t="shared" ref="E56" si="0">(B56-0.0164)/0.0093</f>
         <v>-1.763440860215054</v>
       </c>
-      <c r="F56" s="58"/>
+      <c r="F56" s="56"/>
       <c r="H56" s="18"/>
       <c r="I56" s="27"/>
       <c r="J56" s="18"/>
@@ -16616,15 +16656,15 @@
       <c r="B57" s="6">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="C57" s="76">
+      <c r="C57" s="49">
         <v>5</v>
       </c>
-      <c r="D57" s="76"/>
-      <c r="E57" s="57">
+      <c r="D57" s="49"/>
+      <c r="E57" s="55">
         <f>(B57-0.0164)/0.0093</f>
         <v>2.0000000000000004</v>
       </c>
-      <c r="F57" s="58"/>
+      <c r="F57" s="56"/>
       <c r="H57" s="18">
         <f>C57/1000000</f>
         <v>5.0000000000000004E-6</v>
@@ -16645,10 +16685,10 @@
       <c r="B58" s="6">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="C58" s="76">
+      <c r="C58" s="49">
         <v>10</v>
       </c>
-      <c r="D58" s="76"/>
+      <c r="D58" s="49"/>
       <c r="E58" s="50">
         <f t="shared" ref="E58:E62" si="1">(B58-0.0164)/0.0093</f>
         <v>7.1612903225806468</v>
@@ -16672,10 +16712,10 @@
         <v>36</v>
       </c>
       <c r="B59" s="6"/>
-      <c r="C59" s="76">
+      <c r="C59" s="49">
         <v>25</v>
       </c>
-      <c r="D59" s="76"/>
+      <c r="D59" s="49"/>
       <c r="E59" s="50">
         <f t="shared" si="1"/>
         <v>-1.763440860215054</v>
@@ -16692,10 +16732,10 @@
       <c r="B60" s="6">
         <v>0.48499999999999999</v>
       </c>
-      <c r="C60" s="76">
+      <c r="C60" s="49">
         <v>50</v>
       </c>
-      <c r="D60" s="76"/>
+      <c r="D60" s="49"/>
       <c r="E60" s="50">
         <f t="shared" si="1"/>
         <v>50.387096774193552</v>
@@ -16721,10 +16761,10 @@
       <c r="B61" s="6">
         <v>0.96499999999999997</v>
       </c>
-      <c r="C61" s="76">
+      <c r="C61" s="49">
         <v>100</v>
       </c>
-      <c r="D61" s="76"/>
+      <c r="D61" s="49"/>
       <c r="E61" s="50">
         <f t="shared" si="1"/>
         <v>102.00000000000001</v>
@@ -16750,15 +16790,15 @@
       <c r="B62" s="8">
         <v>1.8340000000000001</v>
       </c>
-      <c r="C62" s="52">
+      <c r="C62" s="61">
         <v>200</v>
       </c>
-      <c r="D62" s="53"/>
-      <c r="E62" s="54">
+      <c r="D62" s="62"/>
+      <c r="E62" s="63">
         <f t="shared" si="1"/>
         <v>195.44086021505379</v>
       </c>
-      <c r="F62" s="55"/>
+      <c r="F62" s="64"/>
       <c r="H62" s="19">
         <f>C62/1000000</f>
         <v>2.0000000000000001E-4</v>
@@ -16779,12 +16819,12 @@
       <c r="B63" s="9">
         <v>1.0999999999999999E-2</v>
       </c>
-      <c r="C63" s="72"/>
-      <c r="D63" s="73"/>
-      <c r="E63" s="74">
+      <c r="C63" s="65"/>
+      <c r="D63" s="66"/>
+      <c r="E63" s="67">
         <v>0</v>
       </c>
-      <c r="F63" s="75"/>
+      <c r="F63" s="68"/>
       <c r="H63" s="18">
         <f t="shared" ref="H63:H70" si="4">E63/1000000</f>
         <v>0</v>
@@ -16805,12 +16845,12 @@
       <c r="B64" s="6">
         <v>2E-3</v>
       </c>
-      <c r="C64" s="48"/>
-      <c r="D64" s="56"/>
-      <c r="E64" s="57">
+      <c r="C64" s="59"/>
+      <c r="D64" s="60"/>
+      <c r="E64" s="55">
         <v>0</v>
       </c>
-      <c r="F64" s="58"/>
+      <c r="F64" s="56"/>
       <c r="H64" s="18">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -16831,12 +16871,12 @@
       <c r="B65" s="6">
         <v>2E-3</v>
       </c>
-      <c r="C65" s="48"/>
-      <c r="D65" s="56"/>
-      <c r="E65" s="57">
+      <c r="C65" s="59"/>
+      <c r="D65" s="60"/>
+      <c r="E65" s="55">
         <v>0</v>
       </c>
-      <c r="F65" s="58"/>
+      <c r="F65" s="56"/>
       <c r="H65" s="18">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -16857,12 +16897,12 @@
       <c r="B66" s="6">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="C66" s="48"/>
-      <c r="D66" s="56"/>
-      <c r="E66" s="57">
+      <c r="C66" s="59"/>
+      <c r="D66" s="60"/>
+      <c r="E66" s="55">
         <v>0</v>
       </c>
-      <c r="F66" s="58"/>
+      <c r="F66" s="56"/>
       <c r="H66" s="18">
         <f t="shared" si="4"/>
         <v>0</v>
@@ -16883,13 +16923,13 @@
       <c r="B67" s="6">
         <v>0.109</v>
       </c>
-      <c r="C67" s="48"/>
-      <c r="D67" s="56"/>
-      <c r="E67" s="57">
+      <c r="C67" s="59"/>
+      <c r="D67" s="60"/>
+      <c r="E67" s="55">
         <f t="shared" ref="E67:E70" si="7">(B67-0.0164)/0.0093</f>
         <v>9.9569892473118298</v>
       </c>
-      <c r="F67" s="58"/>
+      <c r="F67" s="56"/>
       <c r="H67" s="18">
         <f t="shared" si="4"/>
         <v>9.9569892473118294E-6</v>
@@ -16910,13 +16950,13 @@
       <c r="B68" s="6">
         <v>0.36</v>
       </c>
-      <c r="C68" s="48"/>
-      <c r="D68" s="56"/>
-      <c r="E68" s="57">
+      <c r="C68" s="59"/>
+      <c r="D68" s="60"/>
+      <c r="E68" s="55">
         <f t="shared" si="7"/>
         <v>36.946236559139784</v>
       </c>
-      <c r="F68" s="58"/>
+      <c r="F68" s="56"/>
       <c r="H68" s="18">
         <f t="shared" si="4"/>
         <v>3.6946236559139785E-5</v>
@@ -16937,13 +16977,13 @@
       <c r="B69" s="6">
         <v>0.91300000000000003</v>
       </c>
-      <c r="C69" s="48"/>
-      <c r="D69" s="56"/>
-      <c r="E69" s="57">
+      <c r="C69" s="59"/>
+      <c r="D69" s="60"/>
+      <c r="E69" s="55">
         <f t="shared" si="7"/>
         <v>96.408602150537646</v>
       </c>
-      <c r="F69" s="58"/>
+      <c r="F69" s="56"/>
       <c r="H69" s="18">
         <f t="shared" si="4"/>
         <v>9.6408602150537646E-5</v>
@@ -16964,13 +17004,13 @@
       <c r="B70" s="8">
         <v>4.7E-2</v>
       </c>
-      <c r="C70" s="52"/>
-      <c r="D70" s="59"/>
-      <c r="E70" s="60">
+      <c r="C70" s="61"/>
+      <c r="D70" s="69"/>
+      <c r="E70" s="57">
         <f t="shared" si="7"/>
         <v>3.2903225806451615</v>
       </c>
-      <c r="F70" s="61"/>
+      <c r="F70" s="58"/>
       <c r="H70" s="18">
         <f t="shared" si="4"/>
         <v>3.2903225806451615E-6</v>
@@ -17055,11 +17095,11 @@
         <v>0.5</v>
       </c>
       <c r="D101" s="11"/>
-      <c r="E101" s="68">
+      <c r="E101" s="53">
         <f>(B101+0.0049)/0.0204</f>
         <v>0.28921568627450978</v>
       </c>
-      <c r="F101" s="69"/>
+      <c r="F101" s="54"/>
       <c r="I101" s="16">
         <f t="shared" ref="I101:I106" si="8">C101/1000000</f>
         <v>4.9999999999999998E-7</v>
@@ -17084,11 +17124,11 @@
         <v>1</v>
       </c>
       <c r="D102" s="13"/>
-      <c r="E102" s="57">
+      <c r="E102" s="55">
         <f t="shared" ref="E102:E114" si="10">(B102+0.0049)/0.0204</f>
         <v>1.0245098039215685</v>
       </c>
-      <c r="F102" s="58"/>
+      <c r="F102" s="56"/>
       <c r="I102" s="18">
         <f t="shared" si="8"/>
         <v>9.9999999999999995E-7</v>
@@ -17113,11 +17153,11 @@
         <v>5</v>
       </c>
       <c r="D103" s="13"/>
-      <c r="E103" s="57">
+      <c r="E103" s="55">
         <f t="shared" si="10"/>
         <v>4.6029411764705879</v>
       </c>
-      <c r="F103" s="58"/>
+      <c r="F103" s="56"/>
       <c r="I103" s="18">
         <f t="shared" si="8"/>
         <v>5.0000000000000004E-6</v>
@@ -17142,11 +17182,11 @@
         <v>10</v>
       </c>
       <c r="D104" s="13"/>
-      <c r="E104" s="57">
+      <c r="E104" s="55">
         <f t="shared" si="10"/>
         <v>10.877450980392155</v>
       </c>
-      <c r="F104" s="58"/>
+      <c r="F104" s="56"/>
       <c r="I104" s="18">
         <f t="shared" si="8"/>
         <v>1.0000000000000001E-5</v>
@@ -17171,11 +17211,11 @@
         <v>25</v>
       </c>
       <c r="D105" s="33"/>
-      <c r="E105" s="57">
+      <c r="E105" s="55">
         <f t="shared" si="10"/>
         <v>24.799019607843135</v>
       </c>
-      <c r="F105" s="58"/>
+      <c r="F105" s="56"/>
       <c r="I105" s="18">
         <f t="shared" si="8"/>
         <v>2.5000000000000001E-5</v>
@@ -17200,11 +17240,11 @@
         <v>50</v>
       </c>
       <c r="D106" s="15"/>
-      <c r="E106" s="60">
+      <c r="E106" s="57">
         <f t="shared" si="10"/>
         <v>37.446078431372548</v>
       </c>
-      <c r="F106" s="61"/>
+      <c r="F106" s="58"/>
       <c r="I106" s="19">
         <f t="shared" si="8"/>
         <v>5.0000000000000002E-5</v>
@@ -17225,13 +17265,13 @@
       <c r="B107" s="9">
         <v>0</v>
       </c>
-      <c r="C107" s="72"/>
-      <c r="D107" s="73"/>
-      <c r="E107" s="74">
+      <c r="C107" s="65"/>
+      <c r="D107" s="66"/>
+      <c r="E107" s="67">
         <f t="shared" si="10"/>
         <v>0.24019607843137253</v>
       </c>
-      <c r="F107" s="75"/>
+      <c r="F107" s="68"/>
       <c r="I107" s="18">
         <f>E107/1000000</f>
         <v>2.4019607843137255E-7</v>
@@ -17252,13 +17292,13 @@
       <c r="B108" s="6">
         <v>0</v>
       </c>
-      <c r="C108" s="48"/>
-      <c r="D108" s="56"/>
-      <c r="E108" s="57">
+      <c r="C108" s="59"/>
+      <c r="D108" s="60"/>
+      <c r="E108" s="55">
         <f t="shared" si="10"/>
         <v>0.24019607843137253</v>
       </c>
-      <c r="F108" s="58"/>
+      <c r="F108" s="56"/>
       <c r="I108" s="18">
         <f t="shared" ref="I108:I114" si="12">E108/1000000</f>
         <v>2.4019607843137255E-7</v>
@@ -17279,13 +17319,13 @@
       <c r="B109" s="6">
         <v>0</v>
       </c>
-      <c r="C109" s="48"/>
-      <c r="D109" s="56"/>
-      <c r="E109" s="57">
+      <c r="C109" s="59"/>
+      <c r="D109" s="60"/>
+      <c r="E109" s="55">
         <f t="shared" si="10"/>
         <v>0.24019607843137253</v>
       </c>
-      <c r="F109" s="58"/>
+      <c r="F109" s="56"/>
       <c r="I109" s="18">
         <f t="shared" si="12"/>
         <v>2.4019607843137255E-7</v>
@@ -17306,13 +17346,13 @@
       <c r="B110" s="6">
         <v>0</v>
       </c>
-      <c r="C110" s="48"/>
-      <c r="D110" s="56"/>
-      <c r="E110" s="57">
+      <c r="C110" s="59"/>
+      <c r="D110" s="60"/>
+      <c r="E110" s="55">
         <f t="shared" si="10"/>
         <v>0.24019607843137253</v>
       </c>
-      <c r="F110" s="58"/>
+      <c r="F110" s="56"/>
       <c r="I110" s="18">
         <f t="shared" si="12"/>
         <v>2.4019607843137255E-7</v>
@@ -17333,13 +17373,13 @@
       <c r="B111" s="6">
         <v>1.4E-2</v>
       </c>
-      <c r="C111" s="48"/>
-      <c r="D111" s="56"/>
-      <c r="E111" s="57">
+      <c r="C111" s="59"/>
+      <c r="D111" s="60"/>
+      <c r="E111" s="55">
         <f t="shared" si="10"/>
         <v>0.92647058823529405</v>
       </c>
-      <c r="F111" s="58"/>
+      <c r="F111" s="56"/>
       <c r="I111" s="18">
         <f t="shared" si="12"/>
         <v>9.2647058823529408E-7</v>
@@ -17360,13 +17400,13 @@
       <c r="B112" s="6">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="C112" s="48"/>
-      <c r="D112" s="56"/>
-      <c r="E112" s="57">
+      <c r="C112" s="59"/>
+      <c r="D112" s="60"/>
+      <c r="E112" s="55">
         <f t="shared" si="10"/>
         <v>0.68137254901960775</v>
       </c>
-      <c r="F112" s="58"/>
+      <c r="F112" s="56"/>
       <c r="I112" s="18">
         <f t="shared" si="12"/>
         <v>6.8137254901960776E-7</v>
@@ -17387,13 +17427,13 @@
       <c r="B113" s="6">
         <v>3.9E-2</v>
       </c>
-      <c r="C113" s="48"/>
-      <c r="D113" s="56"/>
-      <c r="E113" s="57">
+      <c r="C113" s="59"/>
+      <c r="D113" s="60"/>
+      <c r="E113" s="55">
         <f t="shared" si="10"/>
         <v>2.1519607843137254</v>
       </c>
-      <c r="F113" s="58"/>
+      <c r="F113" s="56"/>
       <c r="I113" s="18">
         <f t="shared" si="12"/>
         <v>2.1519607843137253E-6</v>
@@ -17414,13 +17454,13 @@
       <c r="B114" s="8">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="C114" s="52"/>
-      <c r="D114" s="59"/>
-      <c r="E114" s="60">
+      <c r="C114" s="61"/>
+      <c r="D114" s="69"/>
+      <c r="E114" s="57">
         <f t="shared" si="10"/>
         <v>0.53431372549019607</v>
       </c>
-      <c r="F114" s="61"/>
+      <c r="F114" s="58"/>
       <c r="I114" s="18">
         <f t="shared" si="12"/>
         <v>5.3431372549019611E-7</v>
@@ -17452,16 +17492,16 @@
       </c>
     </row>
     <row r="120" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A120" s="70" t="s">
+      <c r="A120" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="B120" s="70"/>
-      <c r="C120" s="70"/>
-      <c r="D120" s="70"/>
-      <c r="E120" s="70"/>
-      <c r="F120" s="70"/>
-      <c r="G120" s="70"/>
-      <c r="H120" s="70"/>
+      <c r="B120" s="48"/>
+      <c r="C120" s="48"/>
+      <c r="D120" s="48"/>
+      <c r="E120" s="48"/>
+      <c r="F120" s="48"/>
+      <c r="G120" s="48"/>
+      <c r="H120" s="48"/>
     </row>
     <row r="121" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I121" s="16" t="s">
@@ -17507,14 +17547,14 @@
       <c r="B123" s="4">
         <v>0</v>
       </c>
-      <c r="C123" s="62">
+      <c r="C123" s="70">
         <v>2.5</v>
       </c>
-      <c r="D123" s="63"/>
-      <c r="E123" s="68">
+      <c r="D123" s="72"/>
+      <c r="E123" s="53">
         <v>0</v>
       </c>
-      <c r="F123" s="69"/>
+      <c r="F123" s="54"/>
       <c r="G123" s="35"/>
       <c r="I123" s="16">
         <f t="shared" ref="I123:I130" si="15">C123/1000000</f>
@@ -17536,10 +17576,10 @@
       <c r="B124" s="2">
         <v>1E-3</v>
       </c>
-      <c r="C124" s="66">
+      <c r="C124" s="76">
         <v>5</v>
       </c>
-      <c r="D124" s="67"/>
+      <c r="D124" s="77"/>
       <c r="E124" s="50">
         <f t="shared" ref="E124:E138" si="16">(B124+0.0067)/0.0019</f>
         <v>4.0526315789473681</v>
@@ -17566,10 +17606,10 @@
       <c r="B125" s="6">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="C125" s="48">
+      <c r="C125" s="59">
         <v>10</v>
       </c>
-      <c r="D125" s="49"/>
+      <c r="D125" s="75"/>
       <c r="E125" s="50">
         <f t="shared" si="16"/>
         <v>7.7368421052631584</v>
@@ -17596,10 +17636,10 @@
       <c r="B126" s="6">
         <v>4.1000000000000002E-2</v>
       </c>
-      <c r="C126" s="48">
+      <c r="C126" s="59">
         <v>25</v>
       </c>
-      <c r="D126" s="49"/>
+      <c r="D126" s="75"/>
       <c r="E126" s="50">
         <f t="shared" si="16"/>
         <v>25.105263157894736</v>
@@ -17626,10 +17666,10 @@
       <c r="B127" s="6">
         <v>8.3000000000000004E-2</v>
       </c>
-      <c r="C127" s="48">
+      <c r="C127" s="59">
         <v>50</v>
       </c>
-      <c r="D127" s="49"/>
+      <c r="D127" s="75"/>
       <c r="E127" s="50">
         <f t="shared" si="16"/>
         <v>47.210526315789473</v>
@@ -17656,10 +17696,10 @@
       <c r="B128" s="6">
         <v>0.17499999999999999</v>
       </c>
-      <c r="C128" s="48">
+      <c r="C128" s="59">
         <v>100</v>
       </c>
-      <c r="D128" s="49"/>
+      <c r="D128" s="75"/>
       <c r="E128" s="50">
         <f t="shared" si="16"/>
         <v>95.631578947368425</v>
@@ -17686,10 +17726,10 @@
       <c r="B129" s="6">
         <v>0.375</v>
       </c>
-      <c r="C129" s="48">
+      <c r="C129" s="59">
         <v>200</v>
       </c>
-      <c r="D129" s="49"/>
+      <c r="D129" s="75"/>
       <c r="E129" s="50">
         <f t="shared" si="16"/>
         <v>200.89473684210526</v>
@@ -17716,15 +17756,15 @@
       <c r="B130" s="8">
         <v>0.91500000000000004</v>
       </c>
-      <c r="C130" s="52">
+      <c r="C130" s="61">
         <v>500</v>
       </c>
-      <c r="D130" s="53"/>
-      <c r="E130" s="54">
+      <c r="D130" s="62"/>
+      <c r="E130" s="63">
         <f t="shared" si="16"/>
         <v>485.1052631578948</v>
       </c>
-      <c r="F130" s="55"/>
+      <c r="F130" s="64"/>
       <c r="G130" s="35"/>
       <c r="I130" s="19">
         <f t="shared" si="15"/>
@@ -17746,13 +17786,13 @@
       <c r="B131" s="9">
         <v>1.0999999999999999E-2</v>
       </c>
-      <c r="C131" s="72"/>
+      <c r="C131" s="65"/>
       <c r="D131" s="78"/>
-      <c r="E131" s="64">
+      <c r="E131" s="73">
         <f t="shared" si="16"/>
         <v>9.3157894736842106</v>
       </c>
-      <c r="F131" s="65"/>
+      <c r="F131" s="74"/>
       <c r="G131" s="35"/>
       <c r="I131" s="18">
         <f>E131/1000000</f>
@@ -17774,8 +17814,8 @@
       <c r="B132" s="6">
         <v>0</v>
       </c>
-      <c r="C132" s="48"/>
-      <c r="D132" s="49"/>
+      <c r="C132" s="59"/>
+      <c r="D132" s="75"/>
       <c r="E132" s="50">
         <v>0</v>
       </c>
@@ -17801,8 +17841,8 @@
       <c r="B133" s="6">
         <v>0</v>
       </c>
-      <c r="C133" s="48"/>
-      <c r="D133" s="49"/>
+      <c r="C133" s="59"/>
+      <c r="D133" s="75"/>
       <c r="E133" s="50">
         <v>0</v>
       </c>
@@ -17828,8 +17868,8 @@
       <c r="B134" s="6">
         <v>0</v>
       </c>
-      <c r="C134" s="48"/>
-      <c r="D134" s="49"/>
+      <c r="C134" s="59"/>
+      <c r="D134" s="75"/>
       <c r="E134" s="50">
         <v>0</v>
       </c>
@@ -17855,8 +17895,8 @@
       <c r="B135" s="6">
         <v>0</v>
       </c>
-      <c r="C135" s="48"/>
-      <c r="D135" s="49"/>
+      <c r="C135" s="59"/>
+      <c r="D135" s="75"/>
       <c r="E135" s="50">
         <v>0</v>
       </c>
@@ -17882,8 +17922,8 @@
       <c r="B136" s="6">
         <v>1.7999999999999999E-2</v>
       </c>
-      <c r="C136" s="48"/>
-      <c r="D136" s="49"/>
+      <c r="C136" s="59"/>
+      <c r="D136" s="75"/>
       <c r="E136" s="50">
         <f t="shared" si="16"/>
         <v>13</v>
@@ -17910,8 +17950,8 @@
       <c r="B137" s="6">
         <v>2.8000000000000001E-2</v>
       </c>
-      <c r="C137" s="48"/>
-      <c r="D137" s="49"/>
+      <c r="C137" s="59"/>
+      <c r="D137" s="75"/>
       <c r="E137" s="50">
         <f t="shared" si="16"/>
         <v>18.263157894736842</v>
@@ -17938,13 +17978,13 @@
       <c r="B138" s="8">
         <v>2.7E-2</v>
       </c>
-      <c r="C138" s="52"/>
-      <c r="D138" s="53"/>
-      <c r="E138" s="54">
+      <c r="C138" s="61"/>
+      <c r="D138" s="62"/>
+      <c r="E138" s="63">
         <f t="shared" si="16"/>
         <v>17.736842105263158</v>
       </c>
-      <c r="F138" s="55"/>
+      <c r="F138" s="64"/>
       <c r="G138" s="35"/>
       <c r="I138" s="18">
         <f t="shared" si="21"/>
@@ -17961,55 +18001,32 @@
     </row>
   </sheetData>
   <mergeCells count="88">
-    <mergeCell ref="C57:D57"/>
-    <mergeCell ref="E57:F57"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="C55:D55"/>
-    <mergeCell ref="E55:F55"/>
-    <mergeCell ref="C56:D56"/>
-    <mergeCell ref="E56:F56"/>
-    <mergeCell ref="C58:D58"/>
-    <mergeCell ref="E58:F58"/>
-    <mergeCell ref="C59:D59"/>
-    <mergeCell ref="E59:F59"/>
-    <mergeCell ref="C60:D60"/>
-    <mergeCell ref="E60:F60"/>
-    <mergeCell ref="C61:D61"/>
-    <mergeCell ref="E61:F61"/>
-    <mergeCell ref="C62:D62"/>
-    <mergeCell ref="E62:F62"/>
-    <mergeCell ref="C63:D63"/>
-    <mergeCell ref="E63:F63"/>
-    <mergeCell ref="C64:D64"/>
-    <mergeCell ref="E64:F64"/>
-    <mergeCell ref="C65:D65"/>
-    <mergeCell ref="E65:F65"/>
-    <mergeCell ref="C66:D66"/>
-    <mergeCell ref="E66:F66"/>
-    <mergeCell ref="E104:F104"/>
-    <mergeCell ref="C67:D67"/>
-    <mergeCell ref="E67:F67"/>
-    <mergeCell ref="C68:D68"/>
-    <mergeCell ref="E68:F68"/>
-    <mergeCell ref="C69:D69"/>
-    <mergeCell ref="E69:F69"/>
-    <mergeCell ref="C70:D70"/>
-    <mergeCell ref="E70:F70"/>
-    <mergeCell ref="E101:F101"/>
-    <mergeCell ref="E102:F102"/>
-    <mergeCell ref="E103:F103"/>
-    <mergeCell ref="E105:F105"/>
-    <mergeCell ref="E106:F106"/>
-    <mergeCell ref="C107:D107"/>
-    <mergeCell ref="E107:F107"/>
-    <mergeCell ref="C108:D108"/>
-    <mergeCell ref="E108:F108"/>
-    <mergeCell ref="C109:D109"/>
-    <mergeCell ref="E109:F109"/>
-    <mergeCell ref="C110:D110"/>
-    <mergeCell ref="E110:F110"/>
-    <mergeCell ref="C111:D111"/>
-    <mergeCell ref="E111:F111"/>
+    <mergeCell ref="C138:D138"/>
+    <mergeCell ref="E138:F138"/>
+    <mergeCell ref="C135:D135"/>
+    <mergeCell ref="E135:F135"/>
+    <mergeCell ref="C136:D136"/>
+    <mergeCell ref="E136:F136"/>
+    <mergeCell ref="C137:D137"/>
+    <mergeCell ref="E137:F137"/>
+    <mergeCell ref="C132:D132"/>
+    <mergeCell ref="E132:F132"/>
+    <mergeCell ref="C133:D133"/>
+    <mergeCell ref="E133:F133"/>
+    <mergeCell ref="C134:D134"/>
+    <mergeCell ref="E134:F134"/>
+    <mergeCell ref="C129:D129"/>
+    <mergeCell ref="E129:F129"/>
+    <mergeCell ref="C130:D130"/>
+    <mergeCell ref="E130:F130"/>
+    <mergeCell ref="C131:D131"/>
+    <mergeCell ref="E131:F131"/>
+    <mergeCell ref="C126:D126"/>
+    <mergeCell ref="E126:F126"/>
+    <mergeCell ref="C127:D127"/>
+    <mergeCell ref="E127:F127"/>
+    <mergeCell ref="C128:D128"/>
+    <mergeCell ref="E128:F128"/>
     <mergeCell ref="C125:D125"/>
     <mergeCell ref="E125:F125"/>
     <mergeCell ref="C112:D112"/>
@@ -18023,32 +18040,55 @@
     <mergeCell ref="E123:F123"/>
     <mergeCell ref="C124:D124"/>
     <mergeCell ref="E124:F124"/>
-    <mergeCell ref="C126:D126"/>
-    <mergeCell ref="E126:F126"/>
-    <mergeCell ref="C127:D127"/>
-    <mergeCell ref="E127:F127"/>
-    <mergeCell ref="C128:D128"/>
-    <mergeCell ref="E128:F128"/>
-    <mergeCell ref="C129:D129"/>
-    <mergeCell ref="E129:F129"/>
-    <mergeCell ref="C130:D130"/>
-    <mergeCell ref="E130:F130"/>
-    <mergeCell ref="C131:D131"/>
-    <mergeCell ref="E131:F131"/>
-    <mergeCell ref="C132:D132"/>
-    <mergeCell ref="E132:F132"/>
-    <mergeCell ref="C133:D133"/>
-    <mergeCell ref="E133:F133"/>
-    <mergeCell ref="C134:D134"/>
-    <mergeCell ref="E134:F134"/>
-    <mergeCell ref="C138:D138"/>
-    <mergeCell ref="E138:F138"/>
-    <mergeCell ref="C135:D135"/>
-    <mergeCell ref="E135:F135"/>
-    <mergeCell ref="C136:D136"/>
-    <mergeCell ref="E136:F136"/>
-    <mergeCell ref="C137:D137"/>
-    <mergeCell ref="E137:F137"/>
+    <mergeCell ref="C109:D109"/>
+    <mergeCell ref="E109:F109"/>
+    <mergeCell ref="C110:D110"/>
+    <mergeCell ref="E110:F110"/>
+    <mergeCell ref="C111:D111"/>
+    <mergeCell ref="E111:F111"/>
+    <mergeCell ref="E105:F105"/>
+    <mergeCell ref="E106:F106"/>
+    <mergeCell ref="C107:D107"/>
+    <mergeCell ref="E107:F107"/>
+    <mergeCell ref="C108:D108"/>
+    <mergeCell ref="E108:F108"/>
+    <mergeCell ref="E104:F104"/>
+    <mergeCell ref="C67:D67"/>
+    <mergeCell ref="E67:F67"/>
+    <mergeCell ref="C68:D68"/>
+    <mergeCell ref="E68:F68"/>
+    <mergeCell ref="C69:D69"/>
+    <mergeCell ref="E69:F69"/>
+    <mergeCell ref="C70:D70"/>
+    <mergeCell ref="E70:F70"/>
+    <mergeCell ref="E101:F101"/>
+    <mergeCell ref="E102:F102"/>
+    <mergeCell ref="E103:F103"/>
+    <mergeCell ref="C64:D64"/>
+    <mergeCell ref="E64:F64"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="E65:F65"/>
+    <mergeCell ref="C66:D66"/>
+    <mergeCell ref="E66:F66"/>
+    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="E61:F61"/>
+    <mergeCell ref="C62:D62"/>
+    <mergeCell ref="E62:F62"/>
+    <mergeCell ref="C63:D63"/>
+    <mergeCell ref="E63:F63"/>
+    <mergeCell ref="C58:D58"/>
+    <mergeCell ref="E58:F58"/>
+    <mergeCell ref="C59:D59"/>
+    <mergeCell ref="E59:F59"/>
+    <mergeCell ref="C60:D60"/>
+    <mergeCell ref="E60:F60"/>
+    <mergeCell ref="C57:D57"/>
+    <mergeCell ref="E57:F57"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="C55:D55"/>
+    <mergeCell ref="E55:F55"/>
+    <mergeCell ref="C56:D56"/>
+    <mergeCell ref="E56:F56"/>
   </mergeCells>
   <pageMargins left="0.11458333333333333" right="1.0416666666666666E-2" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -18071,16 +18111,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
       <c r="I1" s="1"/>
     </row>
     <row r="2" spans="1:9" s="25" customFormat="1" x14ac:dyDescent="0.25">
@@ -18289,14 +18329,14 @@
         <v>34</v>
       </c>
       <c r="B56" s="4"/>
-      <c r="C56" s="77">
+      <c r="C56" s="52">
         <v>1</v>
       </c>
-      <c r="D56" s="77"/>
-      <c r="E56" s="68">
+      <c r="D56" s="52"/>
+      <c r="E56" s="53">
         <v>0</v>
       </c>
-      <c r="F56" s="69"/>
+      <c r="F56" s="54"/>
       <c r="H56" s="18"/>
       <c r="I56" s="27"/>
       <c r="J56" s="18"/>
@@ -18306,15 +18346,15 @@
         <v>35</v>
       </c>
       <c r="B57" s="6"/>
-      <c r="C57" s="76">
+      <c r="C57" s="49">
         <v>2.5</v>
       </c>
-      <c r="D57" s="76"/>
-      <c r="E57" s="57">
+      <c r="D57" s="49"/>
+      <c r="E57" s="55">
         <f>(B57+0.0048)/0.0096</f>
         <v>0.5</v>
       </c>
-      <c r="F57" s="58"/>
+      <c r="F57" s="56"/>
       <c r="H57" s="18"/>
       <c r="I57" s="27"/>
       <c r="J57" s="18"/>
@@ -18326,15 +18366,15 @@
       <c r="B58" s="6">
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="C58" s="76">
+      <c r="C58" s="49">
         <v>5</v>
       </c>
-      <c r="D58" s="76"/>
-      <c r="E58" s="57">
+      <c r="D58" s="49"/>
+      <c r="E58" s="55">
         <f>(B58+0.0048)/0.0096</f>
         <v>4.25</v>
       </c>
-      <c r="F58" s="58"/>
+      <c r="F58" s="56"/>
       <c r="H58" s="18">
         <f>C58/1000000</f>
         <v>5.0000000000000004E-6</v>
@@ -18355,15 +18395,15 @@
       <c r="B59" s="6">
         <v>0.08</v>
       </c>
-      <c r="C59" s="76">
+      <c r="C59" s="49">
         <v>10</v>
       </c>
-      <c r="D59" s="76"/>
-      <c r="E59" s="57">
+      <c r="D59" s="49"/>
+      <c r="E59" s="55">
         <f t="shared" ref="E59:E62" si="0">(B59+0.0048)/0.0096</f>
         <v>8.8333333333333339</v>
       </c>
-      <c r="F59" s="58"/>
+      <c r="F59" s="56"/>
       <c r="H59" s="18">
         <f>C59/1000000</f>
         <v>1.0000000000000001E-5</v>
@@ -18382,15 +18422,15 @@
         <v>36</v>
       </c>
       <c r="B60" s="6"/>
-      <c r="C60" s="76">
+      <c r="C60" s="49">
         <v>25</v>
       </c>
-      <c r="D60" s="76"/>
-      <c r="E60" s="57">
+      <c r="D60" s="49"/>
+      <c r="E60" s="55">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="F60" s="58"/>
+      <c r="F60" s="56"/>
       <c r="H60" s="18"/>
       <c r="I60" s="18"/>
       <c r="J60" s="21"/>
@@ -18402,15 +18442,15 @@
       <c r="B61" s="6">
         <v>0.48399999999999999</v>
       </c>
-      <c r="C61" s="76">
+      <c r="C61" s="49">
         <v>50</v>
       </c>
-      <c r="D61" s="76"/>
-      <c r="E61" s="57">
+      <c r="D61" s="49"/>
+      <c r="E61" s="55">
         <f t="shared" si="0"/>
         <v>50.916666666666671</v>
       </c>
-      <c r="F61" s="58"/>
+      <c r="F61" s="56"/>
       <c r="H61" s="18">
         <f>C61/1000000</f>
         <v>5.0000000000000002E-5</v>
@@ -18431,15 +18471,15 @@
       <c r="B62" s="6">
         <v>0.97299999999999998</v>
       </c>
-      <c r="C62" s="76">
+      <c r="C62" s="49">
         <v>100</v>
       </c>
-      <c r="D62" s="76"/>
-      <c r="E62" s="57">
+      <c r="D62" s="49"/>
+      <c r="E62" s="55">
         <f t="shared" si="0"/>
         <v>101.85416666666667</v>
       </c>
-      <c r="F62" s="58"/>
+      <c r="F62" s="56"/>
       <c r="H62" s="18">
         <f>C62/1000000</f>
         <v>1E-4</v>
@@ -18460,15 +18500,15 @@
       <c r="B63" s="8">
         <v>1.899</v>
       </c>
-      <c r="C63" s="52">
+      <c r="C63" s="61">
         <v>200</v>
       </c>
-      <c r="D63" s="53"/>
-      <c r="E63" s="60">
+      <c r="D63" s="62"/>
+      <c r="E63" s="57">
         <f t="shared" ref="E63" si="3">(B63+0.0048)/0.0096</f>
         <v>198.3125</v>
       </c>
-      <c r="F63" s="61"/>
+      <c r="F63" s="58"/>
       <c r="H63" s="19">
         <f>C63/1000000</f>
         <v>2.0000000000000001E-4</v>
@@ -18489,13 +18529,13 @@
       <c r="B64" s="9">
         <v>1.25</v>
       </c>
-      <c r="C64" s="72"/>
-      <c r="D64" s="73"/>
-      <c r="E64" s="74">
+      <c r="C64" s="65"/>
+      <c r="D64" s="66"/>
+      <c r="E64" s="67">
         <f t="shared" ref="E64" si="4">(B64+0.0048)/0.0096</f>
         <v>130.70833333333334</v>
       </c>
-      <c r="F64" s="75"/>
+      <c r="F64" s="68"/>
       <c r="H64" s="18">
         <f t="shared" ref="H64:H71" si="5">E64/1000000</f>
         <v>1.3070833333333334E-4</v>
@@ -18516,13 +18556,13 @@
       <c r="B65" s="6">
         <v>1E-3</v>
       </c>
-      <c r="C65" s="48"/>
-      <c r="D65" s="56"/>
-      <c r="E65" s="74">
+      <c r="C65" s="59"/>
+      <c r="D65" s="60"/>
+      <c r="E65" s="67">
         <f t="shared" ref="E65:E71" si="6">(B65+0.0048)/0.0096</f>
         <v>0.60416666666666663</v>
       </c>
-      <c r="F65" s="75"/>
+      <c r="F65" s="68"/>
       <c r="H65" s="18">
         <f t="shared" si="5"/>
         <v>6.0416666666666667E-7</v>
@@ -18543,13 +18583,13 @@
       <c r="B66" s="6">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="C66" s="48"/>
-      <c r="D66" s="56"/>
-      <c r="E66" s="74">
+      <c r="C66" s="59"/>
+      <c r="D66" s="60"/>
+      <c r="E66" s="67">
         <f t="shared" si="6"/>
         <v>1.0208333333333335</v>
       </c>
-      <c r="F66" s="75"/>
+      <c r="F66" s="68"/>
       <c r="H66" s="18">
         <f t="shared" si="5"/>
         <v>1.0208333333333334E-6</v>
@@ -18570,13 +18610,13 @@
       <c r="B67" s="6">
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="C67" s="48"/>
-      <c r="D67" s="56"/>
-      <c r="E67" s="74">
+      <c r="C67" s="59"/>
+      <c r="D67" s="60"/>
+      <c r="E67" s="67">
         <f t="shared" si="6"/>
         <v>1.3333333333333333</v>
       </c>
-      <c r="F67" s="75"/>
+      <c r="F67" s="68"/>
       <c r="H67" s="18">
         <f t="shared" si="5"/>
         <v>1.3333333333333332E-6</v>
@@ -18597,13 +18637,13 @@
       <c r="B68" s="6">
         <v>1.4E-2</v>
       </c>
-      <c r="C68" s="48"/>
-      <c r="D68" s="56"/>
-      <c r="E68" s="74">
+      <c r="C68" s="59"/>
+      <c r="D68" s="60"/>
+      <c r="E68" s="67">
         <f t="shared" si="6"/>
         <v>1.9583333333333335</v>
       </c>
-      <c r="F68" s="75"/>
+      <c r="F68" s="68"/>
       <c r="H68" s="18">
         <f t="shared" si="5"/>
         <v>1.9583333333333334E-6</v>
@@ -18624,13 +18664,13 @@
       <c r="B69" s="6">
         <v>2.4E-2</v>
       </c>
-      <c r="C69" s="48"/>
-      <c r="D69" s="56"/>
-      <c r="E69" s="74">
+      <c r="C69" s="59"/>
+      <c r="D69" s="60"/>
+      <c r="E69" s="67">
         <f t="shared" si="6"/>
         <v>3</v>
       </c>
-      <c r="F69" s="75"/>
+      <c r="F69" s="68"/>
       <c r="H69" s="18">
         <f t="shared" si="5"/>
         <v>3.0000000000000001E-6</v>
@@ -18651,13 +18691,13 @@
       <c r="B70" s="6">
         <v>4.1000000000000002E-2</v>
       </c>
-      <c r="C70" s="48"/>
-      <c r="D70" s="56"/>
-      <c r="E70" s="74">
+      <c r="C70" s="59"/>
+      <c r="D70" s="60"/>
+      <c r="E70" s="67">
         <f t="shared" si="6"/>
         <v>4.7708333333333339</v>
       </c>
-      <c r="F70" s="75"/>
+      <c r="F70" s="68"/>
       <c r="H70" s="18">
         <f t="shared" si="5"/>
         <v>4.7708333333333335E-6</v>
@@ -18678,13 +18718,13 @@
       <c r="B71" s="8">
         <v>0.311</v>
       </c>
-      <c r="C71" s="52"/>
-      <c r="D71" s="59"/>
-      <c r="E71" s="81">
+      <c r="C71" s="61"/>
+      <c r="D71" s="69"/>
+      <c r="E71" s="79">
         <f t="shared" si="6"/>
         <v>32.895833333333336</v>
       </c>
-      <c r="F71" s="82"/>
+      <c r="F71" s="80"/>
       <c r="H71" s="18">
         <f t="shared" si="5"/>
         <v>3.2895833333333338E-5</v>
@@ -18769,11 +18809,11 @@
         <v>0.5</v>
       </c>
       <c r="D102" s="11"/>
-      <c r="E102" s="68">
+      <c r="E102" s="53">
         <f>(B102+0.001)/0.0211</f>
         <v>0.56872037914691942</v>
       </c>
-      <c r="F102" s="69"/>
+      <c r="F102" s="54"/>
       <c r="I102" s="16">
         <f t="shared" ref="I102:I107" si="9">C102/1000000</f>
         <v>4.9999999999999998E-7</v>
@@ -18798,11 +18838,11 @@
         <v>1</v>
       </c>
       <c r="D103" s="13"/>
-      <c r="E103" s="57">
+      <c r="E103" s="55">
         <f t="shared" ref="E103:E107" si="11">(B103+0.001)/0.0211</f>
         <v>1.0426540284360191</v>
       </c>
-      <c r="F103" s="58"/>
+      <c r="F103" s="56"/>
       <c r="I103" s="18">
         <f t="shared" si="9"/>
         <v>9.9999999999999995E-7</v>
@@ -18827,11 +18867,11 @@
         <v>5</v>
       </c>
       <c r="D104" s="13"/>
-      <c r="E104" s="57">
+      <c r="E104" s="55">
         <f t="shared" si="11"/>
         <v>5.0236966824644549</v>
       </c>
-      <c r="F104" s="58"/>
+      <c r="F104" s="56"/>
       <c r="I104" s="18">
         <f t="shared" si="9"/>
         <v>5.0000000000000004E-6</v>
@@ -18856,11 +18896,11 @@
         <v>10</v>
       </c>
       <c r="D105" s="13"/>
-      <c r="E105" s="57">
+      <c r="E105" s="55">
         <f t="shared" si="11"/>
         <v>10.284360189573459</v>
       </c>
-      <c r="F105" s="58"/>
+      <c r="F105" s="56"/>
       <c r="I105" s="18">
         <f t="shared" si="9"/>
         <v>1.0000000000000001E-5</v>
@@ -18885,11 +18925,11 @@
         <v>25</v>
       </c>
       <c r="D106" s="33"/>
-      <c r="E106" s="57">
+      <c r="E106" s="55">
         <f t="shared" si="11"/>
         <v>24.976303317535546</v>
       </c>
-      <c r="F106" s="58"/>
+      <c r="F106" s="56"/>
       <c r="I106" s="19">
         <f t="shared" si="9"/>
         <v>2.5000000000000001E-5</v>
@@ -18914,11 +18954,11 @@
         <v>50</v>
       </c>
       <c r="D107" s="15"/>
-      <c r="E107" s="60">
+      <c r="E107" s="57">
         <f t="shared" si="11"/>
         <v>78.436018957345965</v>
       </c>
-      <c r="F107" s="61"/>
+      <c r="F107" s="58"/>
       <c r="I107" s="18">
         <f t="shared" si="9"/>
         <v>5.0000000000000002E-5</v>
@@ -18939,13 +18979,13 @@
       <c r="B108" s="9">
         <v>0</v>
       </c>
-      <c r="C108" s="72"/>
-      <c r="D108" s="73"/>
-      <c r="E108" s="74">
+      <c r="C108" s="65"/>
+      <c r="D108" s="66"/>
+      <c r="E108" s="67">
         <f t="shared" ref="E108:E115" si="13">(B108+0.001)/0.0211</f>
         <v>4.7393364928909949E-2</v>
       </c>
-      <c r="F108" s="75"/>
+      <c r="F108" s="68"/>
       <c r="I108" s="18">
         <f>E108/1000000</f>
         <v>4.7393364928909948E-8</v>
@@ -18966,13 +19006,13 @@
       <c r="B109" s="6">
         <v>0</v>
       </c>
-      <c r="C109" s="48"/>
-      <c r="D109" s="56"/>
-      <c r="E109" s="57">
+      <c r="C109" s="59"/>
+      <c r="D109" s="60"/>
+      <c r="E109" s="55">
         <f t="shared" si="13"/>
         <v>4.7393364928909949E-2</v>
       </c>
-      <c r="F109" s="58"/>
+      <c r="F109" s="56"/>
       <c r="I109" s="18">
         <f t="shared" ref="I109:I115" si="14">E109/1000000</f>
         <v>4.7393364928909948E-8</v>
@@ -18993,13 +19033,13 @@
       <c r="B110" s="6">
         <v>0</v>
       </c>
-      <c r="C110" s="48"/>
-      <c r="D110" s="56"/>
-      <c r="E110" s="57">
+      <c r="C110" s="59"/>
+      <c r="D110" s="60"/>
+      <c r="E110" s="55">
         <f t="shared" si="13"/>
         <v>4.7393364928909949E-2</v>
       </c>
-      <c r="F110" s="58"/>
+      <c r="F110" s="56"/>
       <c r="I110" s="18">
         <f t="shared" si="14"/>
         <v>4.7393364928909948E-8</v>
@@ -19020,13 +19060,13 @@
       <c r="B111" s="6">
         <v>0</v>
       </c>
-      <c r="C111" s="48"/>
-      <c r="D111" s="56"/>
-      <c r="E111" s="57">
+      <c r="C111" s="59"/>
+      <c r="D111" s="60"/>
+      <c r="E111" s="55">
         <f t="shared" si="13"/>
         <v>4.7393364928909949E-2</v>
       </c>
-      <c r="F111" s="58"/>
+      <c r="F111" s="56"/>
       <c r="I111" s="18">
         <f t="shared" si="14"/>
         <v>4.7393364928909948E-8</v>
@@ -19047,13 +19087,13 @@
       <c r="B112" s="6">
         <v>1.4E-2</v>
       </c>
-      <c r="C112" s="48"/>
-      <c r="D112" s="56"/>
-      <c r="E112" s="57">
+      <c r="C112" s="59"/>
+      <c r="D112" s="60"/>
+      <c r="E112" s="55">
         <f t="shared" si="13"/>
         <v>0.71090047393364919</v>
       </c>
-      <c r="F112" s="58"/>
+      <c r="F112" s="56"/>
       <c r="I112" s="18">
         <f t="shared" si="14"/>
         <v>7.1090047393364923E-7</v>
@@ -19074,13 +19114,13 @@
       <c r="B113" s="6">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="C113" s="48"/>
-      <c r="D113" s="56"/>
-      <c r="E113" s="57">
+      <c r="C113" s="59"/>
+      <c r="D113" s="60"/>
+      <c r="E113" s="55">
         <f t="shared" si="13"/>
         <v>0.47393364928909942</v>
       </c>
-      <c r="F113" s="58"/>
+      <c r="F113" s="56"/>
       <c r="I113" s="18">
         <f t="shared" si="14"/>
         <v>4.7393364928909945E-7</v>
@@ -19101,13 +19141,13 @@
       <c r="B114" s="6">
         <v>3.9E-2</v>
       </c>
-      <c r="C114" s="48"/>
-      <c r="D114" s="56"/>
-      <c r="E114" s="57">
+      <c r="C114" s="59"/>
+      <c r="D114" s="60"/>
+      <c r="E114" s="55">
         <f t="shared" si="13"/>
         <v>1.8957345971563981</v>
       </c>
-      <c r="F114" s="58"/>
+      <c r="F114" s="56"/>
       <c r="I114" s="18">
         <f t="shared" si="14"/>
         <v>1.8957345971563982E-6</v>
@@ -19128,13 +19168,13 @@
       <c r="B115" s="8">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="C115" s="52"/>
-      <c r="D115" s="59"/>
-      <c r="E115" s="60">
+      <c r="C115" s="61"/>
+      <c r="D115" s="69"/>
+      <c r="E115" s="57">
         <f t="shared" si="13"/>
         <v>0.33175355450236965</v>
       </c>
-      <c r="F115" s="61"/>
+      <c r="F115" s="58"/>
       <c r="I115" s="18">
         <f t="shared" si="14"/>
         <v>3.3175355450236965E-7</v>
@@ -19168,16 +19208,16 @@
       <c r="H120" s="24"/>
     </row>
     <row r="121" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A121" s="70" t="s">
+      <c r="A121" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="B121" s="70"/>
-      <c r="C121" s="70"/>
-      <c r="D121" s="70"/>
-      <c r="E121" s="70"/>
-      <c r="F121" s="70"/>
-      <c r="G121" s="70"/>
-      <c r="H121" s="70"/>
+      <c r="B121" s="48"/>
+      <c r="C121" s="48"/>
+      <c r="D121" s="48"/>
+      <c r="E121" s="48"/>
+      <c r="F121" s="48"/>
+      <c r="G121" s="48"/>
+      <c r="H121" s="48"/>
     </row>
     <row r="122" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I122" s="16" t="s">
@@ -19221,14 +19261,14 @@
         <v>56</v>
       </c>
       <c r="B124" s="4"/>
-      <c r="C124" s="62">
+      <c r="C124" s="70">
         <v>2.5</v>
       </c>
-      <c r="D124" s="63"/>
-      <c r="E124" s="68">
+      <c r="D124" s="72"/>
+      <c r="E124" s="53">
         <v>0</v>
       </c>
-      <c r="F124" s="69"/>
+      <c r="F124" s="54"/>
       <c r="G124" s="35"/>
       <c r="I124" s="16">
         <f t="shared" ref="I124:I131" si="17">C124/1000000</f>
@@ -19248,10 +19288,10 @@
         <v>11</v>
       </c>
       <c r="B125" s="2"/>
-      <c r="C125" s="66">
+      <c r="C125" s="76">
         <v>5</v>
       </c>
-      <c r="D125" s="67"/>
+      <c r="D125" s="77"/>
       <c r="E125" s="50">
         <f>(B125+0.0053)/0.0019</f>
         <v>2.7894736842105265</v>
@@ -19278,10 +19318,10 @@
       <c r="B126" s="6">
         <v>2.3E-2</v>
       </c>
-      <c r="C126" s="48">
+      <c r="C126" s="59">
         <v>10</v>
       </c>
-      <c r="D126" s="49"/>
+      <c r="D126" s="75"/>
       <c r="E126" s="50">
         <f t="shared" ref="E126:E131" si="20">(B126+0.0053)/0.0019</f>
         <v>14.894736842105262</v>
@@ -19306,10 +19346,10 @@
         <v>12</v>
       </c>
       <c r="B127" s="6"/>
-      <c r="C127" s="48">
+      <c r="C127" s="59">
         <v>25</v>
       </c>
-      <c r="D127" s="49"/>
+      <c r="D127" s="75"/>
       <c r="E127" s="50">
         <f t="shared" si="20"/>
         <v>2.7894736842105265</v>
@@ -19336,10 +19376,10 @@
       <c r="B128" s="6">
         <v>9.6000000000000002E-2</v>
       </c>
-      <c r="C128" s="48">
+      <c r="C128" s="59">
         <v>50</v>
       </c>
-      <c r="D128" s="49"/>
+      <c r="D128" s="75"/>
       <c r="E128" s="50">
         <f t="shared" si="20"/>
         <v>53.315789473684212</v>
@@ -19366,10 +19406,10 @@
       <c r="B129" s="6">
         <v>0.20499999999999999</v>
       </c>
-      <c r="C129" s="48">
+      <c r="C129" s="59">
         <v>100</v>
       </c>
-      <c r="D129" s="49"/>
+      <c r="D129" s="75"/>
       <c r="E129" s="50">
         <f t="shared" si="20"/>
         <v>110.68421052631578</v>
@@ -19396,10 +19436,10 @@
       <c r="B130" s="6">
         <v>0.39500000000000002</v>
       </c>
-      <c r="C130" s="48">
+      <c r="C130" s="59">
         <v>200</v>
       </c>
-      <c r="D130" s="49"/>
+      <c r="D130" s="75"/>
       <c r="E130" s="50">
         <f t="shared" si="20"/>
         <v>210.68421052631581</v>
@@ -19426,15 +19466,15 @@
       <c r="B131" s="8">
         <v>0.97</v>
       </c>
-      <c r="C131" s="52">
+      <c r="C131" s="61">
         <v>500</v>
       </c>
-      <c r="D131" s="53"/>
-      <c r="E131" s="54">
+      <c r="D131" s="62"/>
+      <c r="E131" s="63">
         <f t="shared" si="20"/>
         <v>513.31578947368416</v>
       </c>
-      <c r="F131" s="55"/>
+      <c r="F131" s="64"/>
       <c r="G131" s="35"/>
       <c r="I131" s="19">
         <f t="shared" si="17"/>
@@ -19456,13 +19496,13 @@
       <c r="B132" s="9">
         <v>1.4E-2</v>
       </c>
-      <c r="C132" s="72"/>
+      <c r="C132" s="65"/>
       <c r="D132" s="78"/>
-      <c r="E132" s="79">
+      <c r="E132" s="81">
         <f t="shared" ref="E132" si="21">(B132+0.0053)/0.0019</f>
         <v>10.157894736842106</v>
       </c>
-      <c r="F132" s="80"/>
+      <c r="F132" s="82"/>
       <c r="G132" s="35"/>
       <c r="I132" s="18">
         <f>E132/1000000</f>
@@ -19484,8 +19524,8 @@
       <c r="B133" s="6">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="C133" s="48"/>
-      <c r="D133" s="49"/>
+      <c r="C133" s="59"/>
+      <c r="D133" s="75"/>
       <c r="E133" s="50">
         <f t="shared" ref="E133" si="24">(B133+0.0053)/0.0019</f>
         <v>7.5263157894736841</v>
@@ -19512,8 +19552,8 @@
       <c r="B134" s="6">
         <v>2E-3</v>
       </c>
-      <c r="C134" s="48"/>
-      <c r="D134" s="49"/>
+      <c r="C134" s="59"/>
+      <c r="D134" s="75"/>
       <c r="E134" s="50">
         <f t="shared" ref="E134:E139" si="25">(B134+0.0053)/0.0019</f>
         <v>3.8421052631578947</v>
@@ -19540,8 +19580,8 @@
       <c r="B135" s="6">
         <v>0</v>
       </c>
-      <c r="C135" s="48"/>
-      <c r="D135" s="49"/>
+      <c r="C135" s="59"/>
+      <c r="D135" s="75"/>
       <c r="E135" s="50">
         <f t="shared" si="25"/>
         <v>2.7894736842105265</v>
@@ -19568,8 +19608,8 @@
       <c r="B136" s="6">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="C136" s="48"/>
-      <c r="D136" s="49"/>
+      <c r="C136" s="59"/>
+      <c r="D136" s="75"/>
       <c r="E136" s="50">
         <f t="shared" si="25"/>
         <v>5.9473684210526319</v>
@@ -19596,8 +19636,8 @@
       <c r="B137" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="C137" s="48"/>
-      <c r="D137" s="49"/>
+      <c r="C137" s="59"/>
+      <c r="D137" s="75"/>
       <c r="E137" s="50">
         <f t="shared" si="25"/>
         <v>15.947368421052632</v>
@@ -19624,8 +19664,8 @@
       <c r="B138" s="6">
         <v>1.2999999999999999E-2</v>
       </c>
-      <c r="C138" s="48"/>
-      <c r="D138" s="49"/>
+      <c r="C138" s="59"/>
+      <c r="D138" s="75"/>
       <c r="E138" s="50">
         <f t="shared" si="25"/>
         <v>9.6315789473684212</v>
@@ -19652,13 +19692,13 @@
       <c r="B139" s="8">
         <v>1.4E-2</v>
       </c>
-      <c r="C139" s="52"/>
-      <c r="D139" s="53"/>
-      <c r="E139" s="54">
+      <c r="C139" s="61"/>
+      <c r="D139" s="62"/>
+      <c r="E139" s="63">
         <f t="shared" si="25"/>
         <v>10.157894736842106</v>
       </c>
-      <c r="F139" s="55"/>
+      <c r="F139" s="64"/>
       <c r="G139" s="35"/>
       <c r="I139" s="18">
         <f t="shared" si="26"/>
@@ -19675,55 +19715,32 @@
     </row>
   </sheetData>
   <mergeCells count="88">
-    <mergeCell ref="C58:D58"/>
-    <mergeCell ref="E58:F58"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="C56:D56"/>
-    <mergeCell ref="E56:F56"/>
-    <mergeCell ref="C57:D57"/>
-    <mergeCell ref="E57:F57"/>
-    <mergeCell ref="C59:D59"/>
-    <mergeCell ref="E59:F59"/>
-    <mergeCell ref="C60:D60"/>
-    <mergeCell ref="E60:F60"/>
-    <mergeCell ref="C61:D61"/>
-    <mergeCell ref="E61:F61"/>
-    <mergeCell ref="C62:D62"/>
-    <mergeCell ref="E62:F62"/>
-    <mergeCell ref="C63:D63"/>
-    <mergeCell ref="E63:F63"/>
-    <mergeCell ref="C64:D64"/>
-    <mergeCell ref="E64:F64"/>
-    <mergeCell ref="C65:D65"/>
-    <mergeCell ref="E65:F65"/>
-    <mergeCell ref="C66:D66"/>
-    <mergeCell ref="E66:F66"/>
-    <mergeCell ref="C67:D67"/>
-    <mergeCell ref="E67:F67"/>
-    <mergeCell ref="E105:F105"/>
-    <mergeCell ref="C68:D68"/>
-    <mergeCell ref="E68:F68"/>
-    <mergeCell ref="C69:D69"/>
-    <mergeCell ref="E69:F69"/>
-    <mergeCell ref="C70:D70"/>
-    <mergeCell ref="E70:F70"/>
-    <mergeCell ref="C71:D71"/>
-    <mergeCell ref="E71:F71"/>
-    <mergeCell ref="E102:F102"/>
-    <mergeCell ref="E103:F103"/>
-    <mergeCell ref="E104:F104"/>
-    <mergeCell ref="E106:F106"/>
-    <mergeCell ref="E107:F107"/>
-    <mergeCell ref="C108:D108"/>
-    <mergeCell ref="E108:F108"/>
-    <mergeCell ref="C109:D109"/>
-    <mergeCell ref="E109:F109"/>
-    <mergeCell ref="C110:D110"/>
-    <mergeCell ref="E110:F110"/>
-    <mergeCell ref="C111:D111"/>
-    <mergeCell ref="E111:F111"/>
-    <mergeCell ref="C112:D112"/>
-    <mergeCell ref="E112:F112"/>
+    <mergeCell ref="C139:D139"/>
+    <mergeCell ref="E139:F139"/>
+    <mergeCell ref="C136:D136"/>
+    <mergeCell ref="E136:F136"/>
+    <mergeCell ref="C137:D137"/>
+    <mergeCell ref="E137:F137"/>
+    <mergeCell ref="C138:D138"/>
+    <mergeCell ref="E138:F138"/>
+    <mergeCell ref="C133:D133"/>
+    <mergeCell ref="E133:F133"/>
+    <mergeCell ref="C134:D134"/>
+    <mergeCell ref="E134:F134"/>
+    <mergeCell ref="C135:D135"/>
+    <mergeCell ref="E135:F135"/>
+    <mergeCell ref="C130:D130"/>
+    <mergeCell ref="E130:F130"/>
+    <mergeCell ref="C131:D131"/>
+    <mergeCell ref="E131:F131"/>
+    <mergeCell ref="C132:D132"/>
+    <mergeCell ref="E132:F132"/>
+    <mergeCell ref="C127:D127"/>
+    <mergeCell ref="E127:F127"/>
+    <mergeCell ref="C128:D128"/>
+    <mergeCell ref="E128:F128"/>
+    <mergeCell ref="C129:D129"/>
+    <mergeCell ref="E129:F129"/>
     <mergeCell ref="C126:D126"/>
     <mergeCell ref="E126:F126"/>
     <mergeCell ref="C113:D113"/>
@@ -19737,32 +19754,55 @@
     <mergeCell ref="E124:F124"/>
     <mergeCell ref="C125:D125"/>
     <mergeCell ref="E125:F125"/>
-    <mergeCell ref="C127:D127"/>
-    <mergeCell ref="E127:F127"/>
-    <mergeCell ref="C128:D128"/>
-    <mergeCell ref="E128:F128"/>
-    <mergeCell ref="C129:D129"/>
-    <mergeCell ref="E129:F129"/>
-    <mergeCell ref="C130:D130"/>
-    <mergeCell ref="E130:F130"/>
-    <mergeCell ref="C131:D131"/>
-    <mergeCell ref="E131:F131"/>
-    <mergeCell ref="C132:D132"/>
-    <mergeCell ref="E132:F132"/>
-    <mergeCell ref="C133:D133"/>
-    <mergeCell ref="E133:F133"/>
-    <mergeCell ref="C134:D134"/>
-    <mergeCell ref="E134:F134"/>
-    <mergeCell ref="C135:D135"/>
-    <mergeCell ref="E135:F135"/>
-    <mergeCell ref="C139:D139"/>
-    <mergeCell ref="E139:F139"/>
-    <mergeCell ref="C136:D136"/>
-    <mergeCell ref="E136:F136"/>
-    <mergeCell ref="C137:D137"/>
-    <mergeCell ref="E137:F137"/>
-    <mergeCell ref="C138:D138"/>
-    <mergeCell ref="E138:F138"/>
+    <mergeCell ref="C110:D110"/>
+    <mergeCell ref="E110:F110"/>
+    <mergeCell ref="C111:D111"/>
+    <mergeCell ref="E111:F111"/>
+    <mergeCell ref="C112:D112"/>
+    <mergeCell ref="E112:F112"/>
+    <mergeCell ref="E106:F106"/>
+    <mergeCell ref="E107:F107"/>
+    <mergeCell ref="C108:D108"/>
+    <mergeCell ref="E108:F108"/>
+    <mergeCell ref="C109:D109"/>
+    <mergeCell ref="E109:F109"/>
+    <mergeCell ref="E105:F105"/>
+    <mergeCell ref="C68:D68"/>
+    <mergeCell ref="E68:F68"/>
+    <mergeCell ref="C69:D69"/>
+    <mergeCell ref="E69:F69"/>
+    <mergeCell ref="C70:D70"/>
+    <mergeCell ref="E70:F70"/>
+    <mergeCell ref="C71:D71"/>
+    <mergeCell ref="E71:F71"/>
+    <mergeCell ref="E102:F102"/>
+    <mergeCell ref="E103:F103"/>
+    <mergeCell ref="E104:F104"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="E65:F65"/>
+    <mergeCell ref="C66:D66"/>
+    <mergeCell ref="E66:F66"/>
+    <mergeCell ref="C67:D67"/>
+    <mergeCell ref="E67:F67"/>
+    <mergeCell ref="C62:D62"/>
+    <mergeCell ref="E62:F62"/>
+    <mergeCell ref="C63:D63"/>
+    <mergeCell ref="E63:F63"/>
+    <mergeCell ref="C64:D64"/>
+    <mergeCell ref="E64:F64"/>
+    <mergeCell ref="C59:D59"/>
+    <mergeCell ref="E59:F59"/>
+    <mergeCell ref="C60:D60"/>
+    <mergeCell ref="E60:F60"/>
+    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="E61:F61"/>
+    <mergeCell ref="C58:D58"/>
+    <mergeCell ref="E58:F58"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="C56:D56"/>
+    <mergeCell ref="E56:F56"/>
+    <mergeCell ref="C57:D57"/>
+    <mergeCell ref="E57:F57"/>
   </mergeCells>
   <pageMargins left="0.11458333333333333" right="1.0416666666666666E-2" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -19785,16 +19825,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
       <c r="I1" s="1"/>
     </row>
     <row r="2" spans="1:9" s="25" customFormat="1" x14ac:dyDescent="0.25">
@@ -20009,14 +20049,14 @@
       <c r="B57" s="6">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="C57" s="76">
+      <c r="C57" s="49">
         <v>1</v>
       </c>
-      <c r="D57" s="76"/>
-      <c r="E57" s="57">
+      <c r="D57" s="49"/>
+      <c r="E57" s="55">
         <v>0</v>
       </c>
-      <c r="F57" s="58"/>
+      <c r="F57" s="56"/>
       <c r="H57" s="18"/>
       <c r="I57" s="27"/>
       <c r="J57" s="18"/>
@@ -20028,15 +20068,15 @@
       <c r="B58" s="6">
         <v>1.7999999999999999E-2</v>
       </c>
-      <c r="C58" s="76">
+      <c r="C58" s="49">
         <v>2.5</v>
       </c>
-      <c r="D58" s="76"/>
-      <c r="E58" s="57">
+      <c r="D58" s="49"/>
+      <c r="E58" s="55">
         <f>(B58-0.0099)/0.0098</f>
         <v>0.82653061224489777</v>
       </c>
-      <c r="F58" s="58"/>
+      <c r="F58" s="56"/>
       <c r="H58" s="18"/>
       <c r="I58" s="27"/>
       <c r="J58" s="18"/>
@@ -20048,15 +20088,15 @@
       <c r="B59" s="6">
         <v>4.2999999999999997E-2</v>
       </c>
-      <c r="C59" s="76">
+      <c r="C59" s="49">
         <v>5</v>
       </c>
-      <c r="D59" s="76"/>
-      <c r="E59" s="57">
+      <c r="D59" s="49"/>
+      <c r="E59" s="55">
         <f t="shared" ref="E59:E64" si="0">(B59-0.0099)/0.0098</f>
         <v>3.3775510204081631</v>
       </c>
-      <c r="F59" s="58"/>
+      <c r="F59" s="56"/>
       <c r="H59" s="18">
         <f>C59/1000000</f>
         <v>5.0000000000000004E-6</v>
@@ -20077,15 +20117,15 @@
       <c r="B60" s="6">
         <v>9.4E-2</v>
       </c>
-      <c r="C60" s="76">
+      <c r="C60" s="49">
         <v>10</v>
       </c>
-      <c r="D60" s="76"/>
-      <c r="E60" s="57">
+      <c r="D60" s="49"/>
+      <c r="E60" s="55">
         <f t="shared" si="0"/>
         <v>8.5816326530612237</v>
       </c>
-      <c r="F60" s="58"/>
+      <c r="F60" s="56"/>
       <c r="H60" s="18">
         <f>C60/1000000</f>
         <v>1.0000000000000001E-5</v>
@@ -20106,15 +20146,15 @@
       <c r="B61" s="6">
         <v>0.25</v>
       </c>
-      <c r="C61" s="76">
+      <c r="C61" s="49">
         <v>25</v>
       </c>
-      <c r="D61" s="76"/>
-      <c r="E61" s="57">
+      <c r="D61" s="49"/>
+      <c r="E61" s="55">
         <f t="shared" si="0"/>
         <v>24.5</v>
       </c>
-      <c r="F61" s="58"/>
+      <c r="F61" s="56"/>
       <c r="H61" s="18"/>
       <c r="I61" s="18"/>
       <c r="J61" s="21"/>
@@ -20126,15 +20166,15 @@
       <c r="B62" s="6">
         <v>0.52</v>
       </c>
-      <c r="C62" s="76">
+      <c r="C62" s="49">
         <v>50</v>
       </c>
-      <c r="D62" s="76"/>
-      <c r="E62" s="57">
+      <c r="D62" s="49"/>
+      <c r="E62" s="55">
         <f t="shared" si="0"/>
         <v>52.051020408163268</v>
       </c>
-      <c r="F62" s="58"/>
+      <c r="F62" s="56"/>
       <c r="H62" s="18">
         <f>C62/1000000</f>
         <v>5.0000000000000002E-5</v>
@@ -20155,15 +20195,15 @@
       <c r="B63" s="6">
         <v>1.028</v>
       </c>
-      <c r="C63" s="76">
+      <c r="C63" s="49">
         <v>100</v>
       </c>
-      <c r="D63" s="76"/>
-      <c r="E63" s="57">
+      <c r="D63" s="49"/>
+      <c r="E63" s="55">
         <f t="shared" si="0"/>
         <v>103.88775510204081</v>
       </c>
-      <c r="F63" s="58"/>
+      <c r="F63" s="56"/>
       <c r="H63" s="18">
         <f>C63/1000000</f>
         <v>1E-4</v>
@@ -20184,15 +20224,15 @@
       <c r="B64" s="8">
         <v>1.95</v>
       </c>
-      <c r="C64" s="52">
+      <c r="C64" s="61">
         <v>200</v>
       </c>
-      <c r="D64" s="53"/>
-      <c r="E64" s="57">
+      <c r="D64" s="62"/>
+      <c r="E64" s="55">
         <f t="shared" si="0"/>
         <v>197.96938775510205</v>
       </c>
-      <c r="F64" s="58"/>
+      <c r="F64" s="56"/>
       <c r="H64" s="19">
         <f>C64/1000000</f>
         <v>2.0000000000000001E-4</v>
@@ -20213,13 +20253,13 @@
       <c r="B65" s="9">
         <v>0.224</v>
       </c>
-      <c r="C65" s="72"/>
-      <c r="D65" s="73"/>
-      <c r="E65" s="57">
+      <c r="C65" s="65"/>
+      <c r="D65" s="66"/>
+      <c r="E65" s="55">
         <f t="shared" ref="E65:E73" si="3">(B65-0.0099)/0.0098</f>
         <v>21.846938775510207</v>
       </c>
-      <c r="F65" s="58"/>
+      <c r="F65" s="56"/>
       <c r="H65" s="18">
         <f t="shared" ref="H65:H73" si="4">E65/1000000</f>
         <v>2.1846938775510207E-5</v>
@@ -20240,13 +20280,13 @@
       <c r="B66" s="6">
         <v>2.9000000000000001E-2</v>
       </c>
-      <c r="C66" s="48"/>
-      <c r="D66" s="56"/>
-      <c r="E66" s="57">
+      <c r="C66" s="59"/>
+      <c r="D66" s="60"/>
+      <c r="E66" s="55">
         <f t="shared" si="3"/>
         <v>1.9489795918367347</v>
       </c>
-      <c r="F66" s="58"/>
+      <c r="F66" s="56"/>
       <c r="H66" s="18">
         <f t="shared" si="4"/>
         <v>1.9489795918367348E-6</v>
@@ -20267,13 +20307,13 @@
       <c r="B67" s="6">
         <v>2.4E-2</v>
       </c>
-      <c r="C67" s="48"/>
-      <c r="D67" s="56"/>
-      <c r="E67" s="57">
+      <c r="C67" s="59"/>
+      <c r="D67" s="60"/>
+      <c r="E67" s="55">
         <f t="shared" si="3"/>
         <v>1.4387755102040816</v>
       </c>
-      <c r="F67" s="58"/>
+      <c r="F67" s="56"/>
       <c r="H67" s="18">
         <f t="shared" si="4"/>
         <v>1.4387755102040816E-6</v>
@@ -20294,13 +20334,13 @@
       <c r="B68" s="6">
         <v>7.9000000000000001E-2</v>
       </c>
-      <c r="C68" s="48"/>
-      <c r="D68" s="56"/>
-      <c r="E68" s="57">
+      <c r="C68" s="59"/>
+      <c r="D68" s="60"/>
+      <c r="E68" s="55">
         <f t="shared" si="3"/>
         <v>7.0510204081632653</v>
       </c>
-      <c r="F68" s="58"/>
+      <c r="F68" s="56"/>
       <c r="H68" s="18">
         <f t="shared" si="4"/>
         <v>7.051020408163265E-6</v>
@@ -20321,13 +20361,13 @@
       <c r="B69" s="6">
         <v>4.1000000000000002E-2</v>
       </c>
-      <c r="C69" s="48"/>
-      <c r="D69" s="56"/>
-      <c r="E69" s="57">
+      <c r="C69" s="59"/>
+      <c r="D69" s="60"/>
+      <c r="E69" s="55">
         <f t="shared" si="3"/>
         <v>3.1734693877551026</v>
       </c>
-      <c r="F69" s="58"/>
+      <c r="F69" s="56"/>
       <c r="H69" s="18">
         <f t="shared" si="4"/>
         <v>3.1734693877551026E-6</v>
@@ -20348,13 +20388,13 @@
       <c r="B70" s="6">
         <v>0.224</v>
       </c>
-      <c r="C70" s="48"/>
-      <c r="D70" s="56"/>
-      <c r="E70" s="57">
+      <c r="C70" s="59"/>
+      <c r="D70" s="60"/>
+      <c r="E70" s="55">
         <f t="shared" si="3"/>
         <v>21.846938775510207</v>
       </c>
-      <c r="F70" s="58"/>
+      <c r="F70" s="56"/>
       <c r="H70" s="18">
         <f t="shared" si="4"/>
         <v>2.1846938775510207E-5</v>
@@ -20375,13 +20415,13 @@
       <c r="B71" s="6">
         <v>0.221</v>
       </c>
-      <c r="C71" s="48"/>
-      <c r="D71" s="56"/>
-      <c r="E71" s="57">
+      <c r="C71" s="59"/>
+      <c r="D71" s="60"/>
+      <c r="E71" s="55">
         <f t="shared" si="3"/>
         <v>21.540816326530614</v>
       </c>
-      <c r="F71" s="58"/>
+      <c r="F71" s="56"/>
       <c r="H71" s="18">
         <f t="shared" si="4"/>
         <v>2.1540816326530614E-5</v>
@@ -20402,13 +20442,13 @@
       <c r="B72" s="6">
         <v>0.11700000000000001</v>
       </c>
-      <c r="C72" s="48"/>
-      <c r="D72" s="56"/>
-      <c r="E72" s="57">
+      <c r="C72" s="59"/>
+      <c r="D72" s="60"/>
+      <c r="E72" s="55">
         <f t="shared" si="3"/>
         <v>10.928571428571429</v>
       </c>
-      <c r="F72" s="58"/>
+      <c r="F72" s="56"/>
       <c r="H72" s="18">
         <f t="shared" si="4"/>
         <v>1.0928571428571429E-5</v>
@@ -20429,13 +20469,13 @@
       <c r="B73" s="6">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="C73" s="48"/>
-      <c r="D73" s="56"/>
-      <c r="E73" s="57">
+      <c r="C73" s="59"/>
+      <c r="D73" s="60"/>
+      <c r="E73" s="55">
         <f t="shared" si="3"/>
         <v>2.5612244897959191</v>
       </c>
-      <c r="F73" s="58"/>
+      <c r="F73" s="56"/>
       <c r="H73" s="18">
         <f t="shared" si="4"/>
         <v>2.5612244897959191E-6</v>
@@ -20520,11 +20560,11 @@
         <v>0.5</v>
       </c>
       <c r="D103" s="11"/>
-      <c r="E103" s="68">
+      <c r="E103" s="53">
         <f>(B103+0.001)/0.0201</f>
         <v>4.975124378109453E-2</v>
       </c>
-      <c r="F103" s="69"/>
+      <c r="F103" s="54"/>
       <c r="I103" s="16">
         <f t="shared" ref="I103:I108" si="7">C103/1000000</f>
         <v>4.9999999999999998E-7</v>
@@ -20549,11 +20589,11 @@
         <v>1</v>
       </c>
       <c r="D104" s="13"/>
-      <c r="E104" s="57">
+      <c r="E104" s="55">
         <f t="shared" ref="E104:E108" si="9">(B104+0.001)/0.0201</f>
         <v>0.54726368159203975</v>
       </c>
-      <c r="F104" s="58"/>
+      <c r="F104" s="56"/>
       <c r="I104" s="18">
         <f t="shared" si="7"/>
         <v>9.9999999999999995E-7</v>
@@ -20578,11 +20618,11 @@
         <v>5</v>
       </c>
       <c r="D105" s="13"/>
-      <c r="E105" s="57">
+      <c r="E105" s="55">
         <f t="shared" si="9"/>
         <v>4.1293532338308463</v>
       </c>
-      <c r="F105" s="58"/>
+      <c r="F105" s="56"/>
       <c r="I105" s="18">
         <f t="shared" si="7"/>
         <v>5.0000000000000004E-6</v>
@@ -20607,11 +20647,11 @@
         <v>10</v>
       </c>
       <c r="D106" s="13"/>
-      <c r="E106" s="57">
+      <c r="E106" s="55">
         <f t="shared" si="9"/>
         <v>10.149253731343284</v>
       </c>
-      <c r="F106" s="58"/>
+      <c r="F106" s="56"/>
       <c r="I106" s="18">
         <f t="shared" si="7"/>
         <v>1.0000000000000001E-5</v>
@@ -20636,11 +20676,11 @@
         <v>25</v>
       </c>
       <c r="D107" s="33"/>
-      <c r="E107" s="57">
+      <c r="E107" s="55">
         <f t="shared" si="9"/>
         <v>24.427860696517413</v>
       </c>
-      <c r="F107" s="58"/>
+      <c r="F107" s="56"/>
       <c r="I107" s="19">
         <f t="shared" si="7"/>
         <v>2.5000000000000001E-5</v>
@@ -20663,11 +20703,11 @@
         <v>50</v>
       </c>
       <c r="D108" s="15"/>
-      <c r="E108" s="60">
+      <c r="E108" s="57">
         <f t="shared" si="9"/>
         <v>4.975124378109453E-2</v>
       </c>
-      <c r="F108" s="61"/>
+      <c r="F108" s="58"/>
       <c r="I108" s="18">
         <f t="shared" si="7"/>
         <v>5.0000000000000002E-5</v>
@@ -20688,13 +20728,13 @@
       <c r="B109" s="9">
         <v>0</v>
       </c>
-      <c r="C109" s="72"/>
-      <c r="D109" s="73"/>
-      <c r="E109" s="74">
+      <c r="C109" s="65"/>
+      <c r="D109" s="66"/>
+      <c r="E109" s="67">
         <f t="shared" ref="E109" si="11">(B109+0.001)/0.0201</f>
         <v>4.975124378109453E-2</v>
       </c>
-      <c r="F109" s="75"/>
+      <c r="F109" s="68"/>
       <c r="I109" s="18">
         <f>E109/1000000</f>
         <v>4.9751243781094531E-8</v>
@@ -20715,13 +20755,13 @@
       <c r="B110" s="6">
         <v>0</v>
       </c>
-      <c r="C110" s="48"/>
-      <c r="D110" s="56"/>
-      <c r="E110" s="57">
+      <c r="C110" s="59"/>
+      <c r="D110" s="60"/>
+      <c r="E110" s="55">
         <f t="shared" ref="E110:E117" si="12">(B110+0.001)/0.0201</f>
         <v>4.975124378109453E-2</v>
       </c>
-      <c r="F110" s="58"/>
+      <c r="F110" s="56"/>
       <c r="I110" s="18">
         <f t="shared" ref="I110:I117" si="13">E110/1000000</f>
         <v>4.9751243781094531E-8</v>
@@ -20742,13 +20782,13 @@
       <c r="B111" s="6">
         <v>0</v>
       </c>
-      <c r="C111" s="48"/>
-      <c r="D111" s="56"/>
-      <c r="E111" s="57">
+      <c r="C111" s="59"/>
+      <c r="D111" s="60"/>
+      <c r="E111" s="55">
         <f t="shared" si="12"/>
         <v>4.975124378109453E-2</v>
       </c>
-      <c r="F111" s="58"/>
+      <c r="F111" s="56"/>
       <c r="I111" s="18">
         <f t="shared" si="13"/>
         <v>4.9751243781094531E-8</v>
@@ -20769,13 +20809,13 @@
       <c r="B112" s="6">
         <v>0</v>
       </c>
-      <c r="C112" s="48"/>
-      <c r="D112" s="56"/>
-      <c r="E112" s="57">
+      <c r="C112" s="59"/>
+      <c r="D112" s="60"/>
+      <c r="E112" s="55">
         <f t="shared" si="12"/>
         <v>4.975124378109453E-2</v>
       </c>
-      <c r="F112" s="58"/>
+      <c r="F112" s="56"/>
       <c r="I112" s="18">
         <f t="shared" si="13"/>
         <v>4.9751243781094531E-8</v>
@@ -20796,13 +20836,13 @@
       <c r="B113" s="6">
         <v>0</v>
       </c>
-      <c r="C113" s="48"/>
-      <c r="D113" s="56"/>
-      <c r="E113" s="57">
+      <c r="C113" s="59"/>
+      <c r="D113" s="60"/>
+      <c r="E113" s="55">
         <f t="shared" si="12"/>
         <v>4.975124378109453E-2</v>
       </c>
-      <c r="F113" s="58"/>
+      <c r="F113" s="56"/>
       <c r="I113" s="18">
         <f t="shared" si="13"/>
         <v>4.9751243781094531E-8</v>
@@ -20823,13 +20863,13 @@
       <c r="B114" s="6">
         <v>2E-3</v>
       </c>
-      <c r="C114" s="48"/>
-      <c r="D114" s="56"/>
-      <c r="E114" s="57">
+      <c r="C114" s="59"/>
+      <c r="D114" s="60"/>
+      <c r="E114" s="55">
         <f t="shared" si="12"/>
         <v>0.1492537313432836</v>
       </c>
-      <c r="F114" s="58"/>
+      <c r="F114" s="56"/>
       <c r="I114" s="18">
         <f t="shared" si="13"/>
         <v>1.492537313432836E-7</v>
@@ -20850,13 +20890,13 @@
       <c r="B115" s="6">
         <v>0.01</v>
       </c>
-      <c r="C115" s="48"/>
-      <c r="D115" s="56"/>
-      <c r="E115" s="57">
+      <c r="C115" s="59"/>
+      <c r="D115" s="60"/>
+      <c r="E115" s="55">
         <f t="shared" si="12"/>
         <v>0.54726368159203975</v>
       </c>
-      <c r="F115" s="58"/>
+      <c r="F115" s="56"/>
       <c r="I115" s="18">
         <f t="shared" si="13"/>
         <v>5.4726368159203972E-7</v>
@@ -20877,13 +20917,13 @@
       <c r="B116" s="6">
         <v>0</v>
       </c>
-      <c r="C116" s="48"/>
-      <c r="D116" s="56"/>
-      <c r="E116" s="57">
+      <c r="C116" s="59"/>
+      <c r="D116" s="60"/>
+      <c r="E116" s="55">
         <f t="shared" si="12"/>
         <v>4.975124378109453E-2</v>
       </c>
-      <c r="F116" s="58"/>
+      <c r="F116" s="56"/>
       <c r="I116" s="18">
         <f t="shared" si="13"/>
         <v>4.9751243781094531E-8</v>
@@ -20904,13 +20944,13 @@
       <c r="B117" s="8">
         <v>0</v>
       </c>
-      <c r="C117" s="52"/>
-      <c r="D117" s="59"/>
-      <c r="E117" s="60">
+      <c r="C117" s="61"/>
+      <c r="D117" s="69"/>
+      <c r="E117" s="57">
         <f t="shared" si="12"/>
         <v>4.975124378109453E-2</v>
       </c>
-      <c r="F117" s="61"/>
+      <c r="F117" s="58"/>
       <c r="I117" s="18">
         <f t="shared" si="13"/>
         <v>4.9751243781094531E-8</v>
@@ -20942,16 +20982,16 @@
       </c>
     </row>
     <row r="122" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A122" s="70" t="s">
+      <c r="A122" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="B122" s="70"/>
-      <c r="C122" s="70"/>
-      <c r="D122" s="70"/>
-      <c r="E122" s="70"/>
-      <c r="F122" s="70"/>
-      <c r="G122" s="70"/>
-      <c r="H122" s="70"/>
+      <c r="B122" s="48"/>
+      <c r="C122" s="48"/>
+      <c r="D122" s="48"/>
+      <c r="E122" s="48"/>
+      <c r="F122" s="48"/>
+      <c r="G122" s="48"/>
+      <c r="H122" s="48"/>
     </row>
     <row r="123" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I123" s="16" t="s">
@@ -20995,14 +21035,14 @@
         <v>56</v>
       </c>
       <c r="B125" s="4"/>
-      <c r="C125" s="62">
+      <c r="C125" s="70">
         <v>2.5</v>
       </c>
-      <c r="D125" s="63"/>
-      <c r="E125" s="68">
+      <c r="D125" s="72"/>
+      <c r="E125" s="53">
         <v>0</v>
       </c>
-      <c r="F125" s="69"/>
+      <c r="F125" s="54"/>
       <c r="G125" s="35"/>
       <c r="I125" s="16">
         <f t="shared" ref="I125:I132" si="16">C125/1000000</f>
@@ -21022,10 +21062,10 @@
         <v>11</v>
       </c>
       <c r="B126" s="2"/>
-      <c r="C126" s="66">
+      <c r="C126" s="76">
         <v>5</v>
       </c>
-      <c r="D126" s="67"/>
+      <c r="D126" s="77"/>
       <c r="E126" s="50">
         <f>(B126-0.0011)/0.0019</f>
         <v>-0.57894736842105265</v>
@@ -21052,10 +21092,10 @@
       <c r="B127" s="6">
         <v>2.1999999999999999E-2</v>
       </c>
-      <c r="C127" s="48">
+      <c r="C127" s="59">
         <v>10</v>
       </c>
-      <c r="D127" s="49"/>
+      <c r="D127" s="75"/>
       <c r="E127" s="50">
         <f t="shared" ref="E127:E141" si="18">(B127-0.0011)/0.0019</f>
         <v>11</v>
@@ -21080,10 +21120,10 @@
         <v>12</v>
       </c>
       <c r="B128" s="6"/>
-      <c r="C128" s="48">
+      <c r="C128" s="59">
         <v>25</v>
       </c>
-      <c r="D128" s="49"/>
+      <c r="D128" s="75"/>
       <c r="E128" s="50">
         <f t="shared" si="18"/>
         <v>-0.57894736842105265</v>
@@ -21110,10 +21150,10 @@
       <c r="B129" s="6">
         <v>0.10199999999999999</v>
       </c>
-      <c r="C129" s="48">
+      <c r="C129" s="59">
         <v>50</v>
       </c>
-      <c r="D129" s="49"/>
+      <c r="D129" s="75"/>
       <c r="E129" s="50">
         <f t="shared" si="18"/>
         <v>53.105263157894733</v>
@@ -21140,10 +21180,10 @@
       <c r="B130" s="6">
         <v>0.19400000000000001</v>
       </c>
-      <c r="C130" s="48">
+      <c r="C130" s="59">
         <v>100</v>
       </c>
-      <c r="D130" s="49"/>
+      <c r="D130" s="75"/>
       <c r="E130" s="50">
         <f t="shared" si="18"/>
         <v>101.5263157894737</v>
@@ -21170,10 +21210,10 @@
       <c r="B131" s="6">
         <v>0.376</v>
       </c>
-      <c r="C131" s="48">
+      <c r="C131" s="59">
         <v>200</v>
       </c>
-      <c r="D131" s="49"/>
+      <c r="D131" s="75"/>
       <c r="E131" s="50">
         <f t="shared" si="18"/>
         <v>197.31578947368422</v>
@@ -21200,15 +21240,15 @@
       <c r="B132" s="8">
         <v>0.96699999999999997</v>
       </c>
-      <c r="C132" s="52">
+      <c r="C132" s="61">
         <v>500</v>
       </c>
-      <c r="D132" s="53"/>
-      <c r="E132" s="54">
+      <c r="D132" s="62"/>
+      <c r="E132" s="63">
         <f t="shared" si="18"/>
         <v>508.36842105263156</v>
       </c>
-      <c r="F132" s="55"/>
+      <c r="F132" s="64"/>
       <c r="G132" s="35"/>
       <c r="I132" s="19">
         <f t="shared" si="16"/>
@@ -21230,13 +21270,13 @@
       <c r="B133" s="9">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="C133" s="72"/>
+      <c r="C133" s="65"/>
       <c r="D133" s="78"/>
-      <c r="E133" s="79">
+      <c r="E133" s="81">
         <f t="shared" si="18"/>
         <v>4.1578947368421044</v>
       </c>
-      <c r="F133" s="80"/>
+      <c r="F133" s="82"/>
       <c r="G133" s="35"/>
       <c r="I133" s="18">
         <f>E133/1000000</f>
@@ -21258,8 +21298,8 @@
       <c r="B134" s="6">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="C134" s="48"/>
-      <c r="D134" s="49"/>
+      <c r="C134" s="59"/>
+      <c r="D134" s="75"/>
       <c r="E134" s="50">
         <f t="shared" si="18"/>
         <v>2.5789473684210527</v>
@@ -21286,8 +21326,8 @@
       <c r="B135" s="6">
         <v>1.0999999999999999E-2</v>
       </c>
-      <c r="C135" s="48"/>
-      <c r="D135" s="49"/>
+      <c r="C135" s="59"/>
+      <c r="D135" s="75"/>
       <c r="E135" s="50">
         <f t="shared" si="18"/>
         <v>5.2105263157894735</v>
@@ -21314,8 +21354,8 @@
       <c r="B136" s="6">
         <v>7.0000000000000001E-3</v>
       </c>
-      <c r="C136" s="48"/>
-      <c r="D136" s="49"/>
+      <c r="C136" s="59"/>
+      <c r="D136" s="75"/>
       <c r="E136" s="50">
         <f t="shared" si="18"/>
         <v>3.1052631578947367</v>
@@ -21342,8 +21382,8 @@
       <c r="B137" s="6">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="C137" s="48"/>
-      <c r="D137" s="49"/>
+      <c r="C137" s="59"/>
+      <c r="D137" s="75"/>
       <c r="E137" s="50">
         <f t="shared" si="18"/>
         <v>2.5789473684210527</v>
@@ -21370,8 +21410,8 @@
       <c r="B138" s="6">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="C138" s="48"/>
-      <c r="D138" s="49"/>
+      <c r="C138" s="59"/>
+      <c r="D138" s="75"/>
       <c r="E138" s="50">
         <f t="shared" si="18"/>
         <v>23.105263157894736</v>
@@ -21398,8 +21438,8 @@
       <c r="B139" s="6">
         <v>3.5999999999999997E-2</v>
       </c>
-      <c r="C139" s="48"/>
-      <c r="D139" s="49"/>
+      <c r="C139" s="59"/>
+      <c r="D139" s="75"/>
       <c r="E139" s="50">
         <f t="shared" si="18"/>
         <v>18.368421052631579</v>
@@ -21426,8 +21466,8 @@
       <c r="B140" s="6">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="C140" s="48"/>
-      <c r="D140" s="49"/>
+      <c r="C140" s="59"/>
+      <c r="D140" s="75"/>
       <c r="E140" s="50">
         <f t="shared" si="18"/>
         <v>13.105263157894736</v>
@@ -21454,13 +21494,13 @@
       <c r="B141" s="8">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="C141" s="52"/>
-      <c r="D141" s="53"/>
-      <c r="E141" s="54">
+      <c r="C141" s="61"/>
+      <c r="D141" s="62"/>
+      <c r="E141" s="63">
         <f t="shared" si="18"/>
         <v>1</v>
       </c>
-      <c r="F141" s="55"/>
+      <c r="F141" s="64"/>
       <c r="I141" s="18">
         <f t="shared" si="22"/>
         <v>9.9999999999999995E-7</v>
@@ -21476,57 +21516,33 @@
     </row>
   </sheetData>
   <mergeCells count="94">
-    <mergeCell ref="C140:D140"/>
-    <mergeCell ref="E140:F140"/>
-    <mergeCell ref="C137:D137"/>
-    <mergeCell ref="E137:F137"/>
-    <mergeCell ref="C138:D138"/>
-    <mergeCell ref="E138:F138"/>
-    <mergeCell ref="C139:D139"/>
-    <mergeCell ref="E139:F139"/>
-    <mergeCell ref="C134:D134"/>
-    <mergeCell ref="E134:F134"/>
-    <mergeCell ref="C135:D135"/>
-    <mergeCell ref="E135:F135"/>
-    <mergeCell ref="C136:D136"/>
-    <mergeCell ref="E136:F136"/>
-    <mergeCell ref="C131:D131"/>
-    <mergeCell ref="E131:F131"/>
-    <mergeCell ref="C132:D132"/>
-    <mergeCell ref="E132:F132"/>
-    <mergeCell ref="C133:D133"/>
-    <mergeCell ref="E133:F133"/>
-    <mergeCell ref="C128:D128"/>
-    <mergeCell ref="E128:F128"/>
-    <mergeCell ref="C129:D129"/>
-    <mergeCell ref="E129:F129"/>
-    <mergeCell ref="C130:D130"/>
-    <mergeCell ref="E130:F130"/>
-    <mergeCell ref="C127:D127"/>
-    <mergeCell ref="E127:F127"/>
-    <mergeCell ref="C114:D114"/>
-    <mergeCell ref="E114:F114"/>
-    <mergeCell ref="C115:D115"/>
-    <mergeCell ref="E115:F115"/>
-    <mergeCell ref="C116:D116"/>
-    <mergeCell ref="E116:F116"/>
-    <mergeCell ref="A122:H122"/>
-    <mergeCell ref="C125:D125"/>
-    <mergeCell ref="E125:F125"/>
-    <mergeCell ref="C126:D126"/>
-    <mergeCell ref="E126:F126"/>
-    <mergeCell ref="C111:D111"/>
-    <mergeCell ref="E111:F111"/>
-    <mergeCell ref="C112:D112"/>
-    <mergeCell ref="E112:F112"/>
-    <mergeCell ref="C113:D113"/>
-    <mergeCell ref="E113:F113"/>
-    <mergeCell ref="E107:F107"/>
-    <mergeCell ref="E108:F108"/>
-    <mergeCell ref="C109:D109"/>
-    <mergeCell ref="E109:F109"/>
-    <mergeCell ref="C110:D110"/>
-    <mergeCell ref="E110:F110"/>
+    <mergeCell ref="C59:D59"/>
+    <mergeCell ref="E59:F59"/>
+    <mergeCell ref="E73:F73"/>
+    <mergeCell ref="C73:D73"/>
+    <mergeCell ref="C141:D141"/>
+    <mergeCell ref="E141:F141"/>
+    <mergeCell ref="C117:D117"/>
+    <mergeCell ref="E117:F117"/>
+    <mergeCell ref="C60:D60"/>
+    <mergeCell ref="E60:F60"/>
+    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="E61:F61"/>
+    <mergeCell ref="C62:D62"/>
+    <mergeCell ref="E62:F62"/>
+    <mergeCell ref="C63:D63"/>
+    <mergeCell ref="E63:F63"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="C57:D57"/>
+    <mergeCell ref="E57:F57"/>
+    <mergeCell ref="C58:D58"/>
+    <mergeCell ref="E58:F58"/>
+    <mergeCell ref="C64:D64"/>
+    <mergeCell ref="E64:F64"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="E65:F65"/>
+    <mergeCell ref="C66:D66"/>
+    <mergeCell ref="E66:F66"/>
     <mergeCell ref="C67:D67"/>
     <mergeCell ref="E67:F67"/>
     <mergeCell ref="C68:D68"/>
@@ -21543,33 +21559,57 @@
     <mergeCell ref="E103:F103"/>
     <mergeCell ref="E104:F104"/>
     <mergeCell ref="E105:F105"/>
-    <mergeCell ref="C64:D64"/>
-    <mergeCell ref="E64:F64"/>
-    <mergeCell ref="C65:D65"/>
-    <mergeCell ref="E65:F65"/>
-    <mergeCell ref="C66:D66"/>
-    <mergeCell ref="E66:F66"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="C57:D57"/>
-    <mergeCell ref="E57:F57"/>
-    <mergeCell ref="C58:D58"/>
-    <mergeCell ref="E58:F58"/>
-    <mergeCell ref="C59:D59"/>
-    <mergeCell ref="E59:F59"/>
-    <mergeCell ref="E73:F73"/>
-    <mergeCell ref="C73:D73"/>
-    <mergeCell ref="C141:D141"/>
-    <mergeCell ref="E141:F141"/>
-    <mergeCell ref="C117:D117"/>
-    <mergeCell ref="E117:F117"/>
-    <mergeCell ref="C60:D60"/>
-    <mergeCell ref="E60:F60"/>
-    <mergeCell ref="C61:D61"/>
-    <mergeCell ref="E61:F61"/>
-    <mergeCell ref="C62:D62"/>
-    <mergeCell ref="E62:F62"/>
-    <mergeCell ref="C63:D63"/>
-    <mergeCell ref="E63:F63"/>
+    <mergeCell ref="E107:F107"/>
+    <mergeCell ref="E108:F108"/>
+    <mergeCell ref="C109:D109"/>
+    <mergeCell ref="E109:F109"/>
+    <mergeCell ref="C110:D110"/>
+    <mergeCell ref="E110:F110"/>
+    <mergeCell ref="C111:D111"/>
+    <mergeCell ref="E111:F111"/>
+    <mergeCell ref="C112:D112"/>
+    <mergeCell ref="E112:F112"/>
+    <mergeCell ref="C113:D113"/>
+    <mergeCell ref="E113:F113"/>
+    <mergeCell ref="C127:D127"/>
+    <mergeCell ref="E127:F127"/>
+    <mergeCell ref="C114:D114"/>
+    <mergeCell ref="E114:F114"/>
+    <mergeCell ref="C115:D115"/>
+    <mergeCell ref="E115:F115"/>
+    <mergeCell ref="C116:D116"/>
+    <mergeCell ref="E116:F116"/>
+    <mergeCell ref="A122:H122"/>
+    <mergeCell ref="C125:D125"/>
+    <mergeCell ref="E125:F125"/>
+    <mergeCell ref="C126:D126"/>
+    <mergeCell ref="E126:F126"/>
+    <mergeCell ref="C128:D128"/>
+    <mergeCell ref="E128:F128"/>
+    <mergeCell ref="C129:D129"/>
+    <mergeCell ref="E129:F129"/>
+    <mergeCell ref="C130:D130"/>
+    <mergeCell ref="E130:F130"/>
+    <mergeCell ref="C131:D131"/>
+    <mergeCell ref="E131:F131"/>
+    <mergeCell ref="C132:D132"/>
+    <mergeCell ref="E132:F132"/>
+    <mergeCell ref="C133:D133"/>
+    <mergeCell ref="E133:F133"/>
+    <mergeCell ref="C134:D134"/>
+    <mergeCell ref="E134:F134"/>
+    <mergeCell ref="C135:D135"/>
+    <mergeCell ref="E135:F135"/>
+    <mergeCell ref="C136:D136"/>
+    <mergeCell ref="E136:F136"/>
+    <mergeCell ref="C140:D140"/>
+    <mergeCell ref="E140:F140"/>
+    <mergeCell ref="C137:D137"/>
+    <mergeCell ref="E137:F137"/>
+    <mergeCell ref="C138:D138"/>
+    <mergeCell ref="E138:F138"/>
+    <mergeCell ref="C139:D139"/>
+    <mergeCell ref="E139:F139"/>
   </mergeCells>
   <pageMargins left="0.11458333333333333" right="1.0416666666666666E-2" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -22472,4 +22512,224 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FB11AC0-5135-4DD2-A5FB-6D266A3E4B2C}">
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="43" t="s">
+        <v>112</v>
+      </c>
+      <c r="D3" s="43" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="84">
+        <v>0.51456029999999997</v>
+      </c>
+      <c r="C4" s="84">
+        <v>1.4198677E-2</v>
+      </c>
+      <c r="D4" s="84">
+        <v>0.90296929999999997</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B5" s="84">
+        <v>2.01386E-2</v>
+      </c>
+      <c r="C5" s="84">
+        <v>2.604468E-3</v>
+      </c>
+      <c r="D5" s="84">
+        <v>0.12944990000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B6" s="84">
+        <v>0.40045619999999998</v>
+      </c>
+      <c r="C6" s="84">
+        <v>7.1953829999999996E-3</v>
+      </c>
+      <c r="D6" s="84">
+        <v>0.32144899999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="B11" s="83" t="s">
+        <v>113</v>
+      </c>
+      <c r="C11" s="83" t="s">
+        <v>112</v>
+      </c>
+      <c r="D11" s="83" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B12" s="84">
+        <v>0.22730737000000001</v>
+      </c>
+      <c r="C12" s="84">
+        <v>6.5395380999999997E-3</v>
+      </c>
+      <c r="D12" s="84">
+        <v>0.91050034999999996</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B13" s="84">
+        <v>0.98818676999999999</v>
+      </c>
+      <c r="C13" s="84">
+        <v>3.0426010900000001E-2</v>
+      </c>
+      <c r="D13" s="84">
+        <v>1.00024501</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="B14" s="84">
+        <v>0.44527673000000001</v>
+      </c>
+      <c r="C14" s="84">
+        <v>8.9557908999999998E-3</v>
+      </c>
+      <c r="D14" s="84">
+        <v>1.00840361</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="B15" s="84">
+        <v>4.620055E-2</v>
+      </c>
+      <c r="C15" s="84">
+        <v>8.9743579999999998E-4</v>
+      </c>
+      <c r="D15" s="84">
+        <v>6.2005400000000002E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B16" s="84">
+        <v>3.7810209999999997E-2</v>
+      </c>
+      <c r="C16" s="84">
+        <v>2.6044685000000001E-3</v>
+      </c>
+      <c r="D16" s="84">
+        <v>9.1376379999999993E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B17" s="84">
+        <v>1.151371E-2</v>
+      </c>
+      <c r="C17" s="84">
+        <v>2.6044685000000001E-3</v>
+      </c>
+      <c r="D17" s="84">
+        <v>0.15664522</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B18" s="84">
+        <v>1.109189E-2</v>
+      </c>
+      <c r="C18" s="84">
+        <v>2.6044685000000001E-3</v>
+      </c>
+      <c r="D18" s="84">
+        <v>0.14032801</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B19" s="84">
+        <v>0.11294683</v>
+      </c>
+      <c r="C19" s="84">
+        <v>1.17862977E-2</v>
+      </c>
+      <c r="D19" s="84">
+        <v>0.13216940999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="84">
+        <v>0.68796553999999999</v>
+      </c>
+      <c r="C20" s="84">
+        <v>2.6044685000000001E-3</v>
+      </c>
+      <c r="D20" s="84">
+        <v>0.51072868999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>